<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 20:12 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
@@ -1769,13 +1769,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46162.79178179398</v>
+        <v>46162.62511512732</v>
       </c>
       <c r="C4" s="5">
-        <v>46183.58133199074</v>
+        <v>46183.414665324075</v>
       </c>
       <c r="D4" s="5">
-        <v>46183.58134738426</v>
+        <v>46183.41468071759</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1822,13 +1822,13 @@
         <v>28</v>
       </c>
       <c r="B5" s="9">
-        <v>46162.79189126157</v>
+        <v>46162.62522459491</v>
       </c>
       <c r="C5" s="9">
-        <v>46183.58129599537</v>
+        <v>46183.414629328705</v>
       </c>
       <c r="D5" s="9">
-        <v>46183.581316400465</v>
+        <v>46183.41464973379</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>29</v>
@@ -1887,13 +1887,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46162.79189434028</v>
+        <v>46162.62522767361</v>
       </c>
       <c r="C6" s="5">
-        <v>46183.58130109953</v>
+        <v>46183.41463443287</v>
       </c>
       <c r="D6" s="5">
-        <v>46183.58131646991</v>
+        <v>46183.41464980324</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1952,13 +1952,13 @@
         <v>36</v>
       </c>
       <c r="B7" s="9">
-        <v>46162.79190123842</v>
+        <v>46162.62523457176</v>
       </c>
       <c r="C7" s="9">
-        <v>46183.58131381945</v>
+        <v>46183.41464715278</v>
       </c>
       <c r="D7" s="9">
-        <v>46183.58133177084</v>
+        <v>46183.41466510417</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>37</v>
@@ -2017,13 +2017,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46162.791904513884</v>
+        <v>46162.62523784723</v>
       </c>
       <c r="C8" s="5">
-        <v>46183.581319641205</v>
+        <v>46183.414652974534</v>
       </c>
       <c r="D8" s="5">
-        <v>46183.58133340278</v>
+        <v>46183.41466673611</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2082,11 +2082,11 @@
         <v>43</v>
       </c>
       <c r="B9" s="9">
-        <v>46162.79178665509</v>
+        <v>46162.62511998843</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="9">
-        <v>46164.64926888889</v>
+        <v>46164.482602222226</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>44</v>
@@ -2129,11 +2129,11 @@
         <v>46</v>
       </c>
       <c r="B10" s="5">
-        <v>46162.7919078125</v>
+        <v>46162.62524114583</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="5">
-        <v>46195.59182194444</v>
+        <v>46195.42515527778</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>47</v>
@@ -2192,11 +2192,11 @@
         <v>54</v>
       </c>
       <c r="B11" s="9">
-        <v>46162.79191291667</v>
+        <v>46162.62524625</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="9">
-        <v>46183.58133586806</v>
+        <v>46183.41466920139</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>55</v>
@@ -2255,11 +2255,11 @@
         <v>58</v>
       </c>
       <c r="B12" s="5">
-        <v>46162.791918055555</v>
+        <v>46162.62525138889</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="5">
-        <v>46183.58133649305</v>
+        <v>46183.414669826394</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>59</v>
@@ -2318,11 +2318,11 @@
         <v>61</v>
       </c>
       <c r="B13" s="9">
-        <v>46162.79192297454</v>
+        <v>46162.625256307874</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="9">
-        <v>46164.68830228009</v>
+        <v>46164.521635613426</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>62</v>
@@ -2381,11 +2381,11 @@
         <v>66</v>
       </c>
       <c r="B14" s="5">
-        <v>46162.791791192125</v>
+        <v>46162.62512452547</v>
       </c>
       <c r="C14" s="6"/>
       <c r="D14" s="5">
-        <v>46164.65944581019</v>
+        <v>46164.49277914352</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>67</v>
@@ -2428,11 +2428,11 @@
         <v>69</v>
       </c>
       <c r="B15" s="9">
-        <v>46162.79193019676</v>
+        <v>46162.62526353009</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="9">
-        <v>46164.688369421296</v>
+        <v>46164.52170275463</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>70</v>
@@ -2491,11 +2491,11 @@
         <v>72</v>
       </c>
       <c r="B16" s="5">
-        <v>46162.7919353125</v>
+        <v>46162.62526864583</v>
       </c>
       <c r="C16" s="6"/>
       <c r="D16" s="5">
-        <v>46164.6883663426</v>
+        <v>46164.521699675926</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>73</v>
@@ -2554,11 +2554,11 @@
         <v>75</v>
       </c>
       <c r="B17" s="9">
-        <v>46162.79194023148</v>
+        <v>46162.625273564816</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46164.68839614584</v>
+        <v>46164.521729479166</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>76</v>
@@ -2617,11 +2617,11 @@
         <v>79</v>
       </c>
       <c r="B18" s="5">
-        <v>46162.791945289355</v>
+        <v>46162.62527862268</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46164.68847915509</v>
+        <v>46164.52181248843</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>80</v>
@@ -2680,11 +2680,11 @@
         <v>85</v>
       </c>
       <c r="B19" s="9">
-        <v>46162.79194956018</v>
+        <v>46162.62528289352</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46164.68847201389</v>
+        <v>46164.52180534722</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>86</v>
@@ -2743,11 +2743,11 @@
         <v>88</v>
       </c>
       <c r="B20" s="5">
-        <v>46162.79195284723</v>
+        <v>46162.625286180555</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46164.688470567125</v>
+        <v>46164.52180390046</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>89</v>
@@ -2806,11 +2806,11 @@
         <v>91</v>
       </c>
       <c r="B21" s="9">
-        <v>46162.79195601852</v>
+        <v>46162.625289351854</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46164.6884696412</v>
+        <v>46164.52180297454</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>92</v>
@@ -2869,11 +2869,11 @@
         <v>94</v>
       </c>
       <c r="B22" s="5">
-        <v>46162.79179634259</v>
+        <v>46162.62512967593</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="5">
-        <v>46164.66016885417</v>
+        <v>46164.4935021875</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>95</v>
@@ -2916,11 +2916,11 @@
         <v>97</v>
       </c>
       <c r="B23" s="9">
-        <v>46162.79196002315</v>
+        <v>46162.62529335648</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="9">
-        <v>46164.68945766204</v>
+        <v>46164.52279099537</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>98</v>
@@ -2979,11 +2979,11 @@
         <v>102</v>
       </c>
       <c r="B24" s="5">
-        <v>46162.791964375</v>
+        <v>46162.625297708335</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="5">
-        <v>46164.689432858795</v>
+        <v>46164.52276619213</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>103</v>
@@ -3038,11 +3038,11 @@
         <v>105</v>
       </c>
       <c r="B25" s="9">
-        <v>46162.79196883102</v>
+        <v>46162.62530216435</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="9">
-        <v>46164.68942958333</v>
+        <v>46164.52276291666</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>106</v>
@@ -3097,11 +3097,11 @@
         <v>108</v>
       </c>
       <c r="B26" s="5">
-        <v>46162.79197329861</v>
+        <v>46162.62530663195</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46169.17544910879</v>
+        <v>46169.00878244213</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>109</v>
@@ -3160,11 +3160,11 @@
         <v>111</v>
       </c>
       <c r="B27" s="9">
-        <v>46162.791977500005</v>
+        <v>46162.62531083333</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="9">
-        <v>46164.68953836805</v>
+        <v>46164.52287170139</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>112</v>
@@ -3219,11 +3219,11 @@
         <v>114</v>
       </c>
       <c r="B28" s="5">
-        <v>46162.79198199074</v>
+        <v>46162.62531532407</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="5">
-        <v>46168.172647141204</v>
+        <v>46168.00598047454</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>115</v>
@@ -3278,11 +3278,11 @@
         <v>117</v>
       </c>
       <c r="B29" s="9">
-        <v>46162.79198653935</v>
+        <v>46162.625319872684</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="9">
-        <v>46164.6896481713</v>
+        <v>46164.52298150463</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>118</v>
@@ -3341,11 +3341,11 @@
         <v>120</v>
       </c>
       <c r="B30" s="5">
-        <v>46162.79199082176</v>
+        <v>46162.62532415509</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="5">
-        <v>46175.170452280094</v>
+        <v>46175.00378561343</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>121</v>
@@ -3400,11 +3400,11 @@
         <v>123</v>
       </c>
       <c r="B31" s="9">
-        <v>46162.791995312495</v>
+        <v>46162.62532864584</v>
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="9">
-        <v>46164.689623750004</v>
+        <v>46164.52295708333</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>124</v>
@@ -3459,11 +3459,11 @@
         <v>126</v>
       </c>
       <c r="B32" s="5">
-        <v>46162.79199990741</v>
+        <v>46162.625333240736</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46164.68961940972</v>
+        <v>46164.52295274306</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>127</v>
@@ -3518,11 +3518,11 @@
         <v>129</v>
       </c>
       <c r="B33" s="9">
-        <v>46162.792004421295</v>
+        <v>46162.62533775463</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="9">
-        <v>46164.68978111111</v>
+        <v>46164.52311444444</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>130</v>
@@ -3581,11 +3581,11 @@
         <v>134</v>
       </c>
       <c r="B34" s="5">
-        <v>46162.79200878472</v>
+        <v>46162.62534211806</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46164.68973819444</v>
+        <v>46164.52307152778</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>135</v>
@@ -3640,11 +3640,11 @@
         <v>137</v>
       </c>
       <c r="B35" s="9">
-        <v>46162.792013391205</v>
+        <v>46162.62534672454</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="9">
-        <v>46164.68973515046</v>
+        <v>46164.523068483795</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>138</v>
@@ -3699,11 +3699,11 @@
         <v>140</v>
       </c>
       <c r="B36" s="5">
-        <v>46162.79201809027</v>
+        <v>46162.625351423616</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46164.689874131946</v>
+        <v>46164.523207465274</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>141</v>
@@ -3762,11 +3762,11 @@
         <v>143</v>
       </c>
       <c r="B37" s="9">
-        <v>46162.79207501157</v>
+        <v>46162.6254083449</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="9">
-        <v>46164.68984363426</v>
+        <v>46164.52317696759</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>87</v>
@@ -3815,11 +3815,11 @@
         <v>145</v>
       </c>
       <c r="B38" s="5">
-        <v>46162.79208025463</v>
+        <v>46162.625413587964</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46164.68984076389</v>
+        <v>46164.52317409722</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>146</v>
@@ -3868,11 +3868,11 @@
         <v>148</v>
       </c>
       <c r="B39" s="9">
-        <v>46162.792085</v>
+        <v>46162.62541833334</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="9">
-        <v>46164.69004553241</v>
+        <v>46164.52337886574</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>149</v>
@@ -3931,11 +3931,11 @@
         <v>153</v>
       </c>
       <c r="B40" s="5">
-        <v>46162.792089166665</v>
+        <v>46162.6254225</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46164.68995886574</v>
+        <v>46164.523292199076</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>93</v>
@@ -3984,11 +3984,11 @@
         <v>155</v>
       </c>
       <c r="B41" s="9">
-        <v>46162.792093599535</v>
+        <v>46162.62542693287</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="9">
-        <v>46164.68995591435</v>
+        <v>46164.523289247685</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>156</v>
@@ -4037,11 +4037,11 @@
         <v>158</v>
       </c>
       <c r="B42" s="5">
-        <v>46162.79210385417</v>
+        <v>46162.6254371875</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46164.68998921296</v>
+        <v>46164.5233225463</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>159</v>
@@ -4090,11 +4090,11 @@
         <v>162</v>
       </c>
       <c r="B43" s="9">
-        <v>46162.79210730324</v>
+        <v>46162.62544063658</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="9">
-        <v>46164.690100057865</v>
+        <v>46164.52343339121</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>163</v>
@@ -4153,11 +4153,11 @@
         <v>165</v>
       </c>
       <c r="B44" s="5">
-        <v>46162.792111180555</v>
+        <v>46162.62544451389</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46164.690157951394</v>
+        <v>46164.52349128472</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>90</v>
@@ -4206,11 +4206,11 @@
         <v>167</v>
       </c>
       <c r="B45" s="9">
-        <v>46162.79211601852</v>
+        <v>46162.62544935185</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="9">
-        <v>46164.69015534723</v>
+        <v>46164.523488680556</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>168</v>
@@ -4259,11 +4259,11 @@
         <v>170</v>
       </c>
       <c r="B46" s="5">
-        <v>46162.791800798615</v>
+        <v>46162.625134131944</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="5">
-        <v>46164.65890277778</v>
+        <v>46164.49223611111</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>171</v>
@@ -4306,11 +4306,11 @@
         <v>173</v>
       </c>
       <c r="B47" s="9">
-        <v>46162.79212121527</v>
+        <v>46162.625454548615</v>
       </c>
       <c r="C47" s="10"/>
       <c r="D47" s="9">
-        <v>46179.19606127315</v>
+        <v>46179.02939460648</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>174</v>
@@ -4369,11 +4369,11 @@
         <v>178</v>
       </c>
       <c r="B48" s="5">
-        <v>46162.79212670139</v>
+        <v>46162.625460034724</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="5">
-        <v>46164.69023148148</v>
+        <v>46164.523564814815</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>179</v>
@@ -4432,11 +4432,11 @@
         <v>182</v>
       </c>
       <c r="B49" s="9">
-        <v>46162.792133090275</v>
+        <v>46162.62546642361</v>
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="9">
-        <v>46164.690227569445</v>
+        <v>46164.52356090277</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>83</v>
@@ -4495,11 +4495,11 @@
         <v>184</v>
       </c>
       <c r="B50" s="5">
-        <v>46162.79214709491</v>
+        <v>46162.625480428236</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46164.69027550926</v>
+        <v>46164.52360884259</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>185</v>
@@ -4558,11 +4558,11 @@
         <v>189</v>
       </c>
       <c r="B51" s="9">
-        <v>46162.792150775465</v>
+        <v>46162.625484108794</v>
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="9">
-        <v>46164.69036847222</v>
+        <v>46164.523701805556</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>190</v>
@@ -4611,11 +4611,11 @@
         <v>192</v>
       </c>
       <c r="B52" s="5">
-        <v>46162.792154849536</v>
+        <v>46162.62548818287</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46164.69036586805</v>
+        <v>46164.52369920139</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>190</v>
@@ -4664,11 +4664,11 @@
         <v>193</v>
       </c>
       <c r="B53" s="9">
-        <v>46162.79215875</v>
+        <v>46162.62549208333</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="9">
-        <v>46164.69036304398</v>
+        <v>46164.52369637731</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>190</v>
@@ -4717,11 +4717,11 @@
         <v>194</v>
       </c>
       <c r="B54" s="5">
-        <v>46162.79216164352</v>
+        <v>46162.62549497685</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46164.690358935186</v>
+        <v>46164.523692268514</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>190</v>
@@ -4770,11 +4770,11 @@
         <v>195</v>
       </c>
       <c r="B55" s="9">
-        <v>46162.7922118287</v>
+        <v>46162.62554516204</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="9">
-        <v>46164.66718020833</v>
+        <v>46164.500513541665</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>196</v>
@@ -4817,11 +4817,11 @@
         <v>198</v>
       </c>
       <c r="B56" s="5">
-        <v>46162.7922200926</v>
+        <v>46162.625553425925</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46164.69048553241</v>
+        <v>46164.52381886574</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>199</v>
@@ -4880,11 +4880,11 @@
         <v>203</v>
       </c>
       <c r="B57" s="9">
-        <v>46162.792225625</v>
+        <v>46162.62555895833</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="9">
-        <v>46164.69055459491</v>
+        <v>46164.52388792824</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>204</v>
@@ -4943,11 +4943,11 @@
         <v>207</v>
       </c>
       <c r="B58" s="5">
-        <v>46162.79223230324</v>
+        <v>46162.625565636576</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46164.690482418984</v>
+        <v>46164.52381575231</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>208</v>
@@ -5006,11 +5006,11 @@
         <v>210</v>
       </c>
       <c r="B59" s="9">
-        <v>46162.79223737269</v>
+        <v>46162.62557070602</v>
       </c>
       <c r="C59" s="10"/>
       <c r="D59" s="9">
-        <v>46164.69055186343</v>
+        <v>46164.52388519676</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>211</v>
@@ -5069,11 +5069,11 @@
         <v>213</v>
       </c>
       <c r="B60" s="5">
-        <v>46162.7922424537</v>
+        <v>46162.62557578704</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46164.6904790625</v>
+        <v>46164.52381239583</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>214</v>
@@ -5132,11 +5132,11 @@
         <v>216</v>
       </c>
       <c r="B61" s="9">
-        <v>46162.792246909725</v>
+        <v>46162.62558024305</v>
       </c>
       <c r="C61" s="10"/>
       <c r="D61" s="9">
-        <v>46164.690549328705</v>
+        <v>46164.52388266203</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>215</v>
@@ -5195,11 +5195,11 @@
         <v>217</v>
       </c>
       <c r="B62" s="5">
-        <v>46162.79225168981</v>
+        <v>46162.62558502315</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46164.66898752315</v>
+        <v>46164.50232085648</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>218</v>
@@ -5242,11 +5242,11 @@
         <v>220</v>
       </c>
       <c r="B63" s="9">
-        <v>46162.792254479165</v>
+        <v>46162.6255878125</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46164.69072508102</v>
+        <v>46164.52405841435</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>221</v>
@@ -5305,11 +5305,11 @@
         <v>224</v>
       </c>
       <c r="B64" s="5">
-        <v>46162.79225922454</v>
+        <v>46162.62559255787</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46164.69068318287</v>
+        <v>46164.5240165162</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>190</v>
@@ -5358,11 +5358,11 @@
         <v>227</v>
       </c>
       <c r="B65" s="9">
-        <v>46162.792265578704</v>
+        <v>46162.62559891204</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="9">
-        <v>46164.69068048611</v>
+        <v>46164.52401381945</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>190</v>
@@ -5411,11 +5411,11 @@
         <v>229</v>
       </c>
       <c r="B66" s="5">
-        <v>46162.79227201389</v>
+        <v>46162.62560534722</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46164.69067753472</v>
+        <v>46164.52401086806</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>190</v>
@@ -5464,11 +5464,11 @@
         <v>232</v>
       </c>
       <c r="B67" s="9">
-        <v>46162.79227828704</v>
+        <v>46162.62561162037</v>
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="9">
-        <v>46164.69067336805</v>
+        <v>46164.52400670139</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>190</v>
@@ -5517,11 +5517,11 @@
         <v>233</v>
       </c>
       <c r="B68" s="5">
-        <v>46162.79232202546</v>
+        <v>46162.625655358795</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46164.69085144676</v>
+        <v>46164.52418478009</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>234</v>
@@ -5580,11 +5580,11 @@
         <v>235</v>
       </c>
       <c r="B69" s="9">
-        <v>46162.79232653935</v>
+        <v>46162.62565987269</v>
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46164.69081627315</v>
+        <v>46164.524149606485</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>190</v>
@@ -5633,11 +5633,11 @@
         <v>238</v>
       </c>
       <c r="B70" s="5">
-        <v>46162.79233265047</v>
+        <v>46162.625665983796</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46164.69081372685</v>
+        <v>46164.52414706019</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>190</v>
@@ -5686,11 +5686,11 @@
         <v>239</v>
       </c>
       <c r="B71" s="9">
-        <v>46162.79233820602</v>
+        <v>46162.625671539354</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46164.690812974535</v>
+        <v>46164.52414630787</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>190</v>
@@ -5739,11 +5739,11 @@
         <v>241</v>
       </c>
       <c r="B72" s="5">
-        <v>46162.79234384259</v>
+        <v>46162.62567717592</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46164.69081170139</v>
+        <v>46164.524145034724</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>190</v>
@@ -5792,11 +5792,11 @@
         <v>242</v>
       </c>
       <c r="B73" s="9">
-        <v>46162.79241414352</v>
+        <v>46162.62574747685</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="9">
-        <v>46164.690976377315</v>
+        <v>46164.52430971064</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>243</v>
@@ -5855,11 +5855,11 @@
         <v>244</v>
       </c>
       <c r="B74" s="5">
-        <v>46162.79242041666</v>
+        <v>46162.62575375</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46164.69094634259</v>
+        <v>46164.52427967593</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>190</v>
@@ -5908,11 +5908,11 @@
         <v>246</v>
       </c>
       <c r="B75" s="9">
-        <v>46162.79243321759</v>
+        <v>46162.625766550926</v>
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46164.69094324074</v>
+        <v>46164.52427657407</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>190</v>
@@ -5961,11 +5961,11 @@
         <v>248</v>
       </c>
       <c r="B76" s="5">
-        <v>46162.79243956019</v>
+        <v>46162.625772893516</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46164.69093616898</v>
+        <v>46164.52426950232</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>190</v>
@@ -6014,11 +6014,11 @@
         <v>250</v>
       </c>
       <c r="B77" s="9">
-        <v>46162.79244651621</v>
+        <v>46162.625779849535</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46164.69093546296</v>
+        <v>46164.5242687963</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>190</v>
@@ -6067,11 +6067,11 @@
         <v>251</v>
       </c>
       <c r="B78" s="5">
-        <v>46162.79247811342</v>
+        <v>46162.625811446764</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46164.670772627316</v>
+        <v>46164.504105960645</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>196</v>
@@ -6114,11 +6114,11 @@
         <v>253</v>
       </c>
       <c r="B79" s="9">
-        <v>46162.792481805554</v>
+        <v>46162.62581513889</v>
       </c>
       <c r="C79" s="10"/>
       <c r="D79" s="9">
-        <v>46171.19919608797</v>
+        <v>46171.032529421296</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>254</v>
@@ -6177,11 +6177,11 @@
         <v>256</v>
       </c>
       <c r="B80" s="5">
-        <v>46162.79248949074</v>
+        <v>46162.62582282408</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46164.691113761575</v>
+        <v>46164.52444709491</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>257</v>
@@ -6240,11 +6240,11 @@
         <v>259</v>
       </c>
       <c r="B81" s="9">
-        <v>46162.79249689815</v>
+        <v>46162.62583023148</v>
       </c>
       <c r="C81" s="10"/>
       <c r="D81" s="9">
-        <v>46164.69111056713</v>
+        <v>46164.52444390046</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>260</v>
@@ -6303,11 +6303,11 @@
         <v>261</v>
       </c>
       <c r="B82" s="5">
-        <v>46162.79250443287</v>
+        <v>46162.6258377662</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46164.69110619213</v>
+        <v>46164.52443952546</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>262</v>
@@ -6366,11 +6366,11 @@
         <v>264</v>
       </c>
       <c r="B83" s="9">
-        <v>46162.79250947917</v>
+        <v>46162.6258428125</v>
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46164.68453591435</v>
+        <v>46164.517869247684</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>265</v>
@@ -6413,11 +6413,11 @@
         <v>267</v>
       </c>
       <c r="B84" s="5">
-        <v>46162.79251295139</v>
+        <v>46162.62584628472</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46164.69124818287</v>
+        <v>46164.524581516205</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>268</v>
@@ -6476,11 +6476,11 @@
         <v>270</v>
       </c>
       <c r="B85" s="9">
-        <v>46162.79252873843</v>
+        <v>46162.625862071756</v>
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46164.69121831018</v>
+        <v>46164.52455164352</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>190</v>
@@ -6529,11 +6529,11 @@
         <v>272</v>
       </c>
       <c r="B86" s="5">
-        <v>46162.792533518514</v>
+        <v>46162.62586685186</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46164.6912157176</v>
+        <v>46164.524549050926</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>190</v>
@@ -6582,11 +6582,11 @@
         <v>273</v>
       </c>
       <c r="B87" s="9">
-        <v>46162.79253825231</v>
+        <v>46162.62587158565</v>
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46164.69121336806</v>
+        <v>46164.52454670139</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>190</v>
@@ -6635,11 +6635,11 @@
         <v>275</v>
       </c>
       <c r="B88" s="5">
-        <v>46162.792543206015</v>
+        <v>46162.62587653935</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46164.691209490746</v>
+        <v>46164.524542824074</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>190</v>
@@ -6688,11 +6688,11 @@
         <v>277</v>
       </c>
       <c r="B89" s="9">
-        <v>46162.792612743055</v>
+        <v>46162.62594607639</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46164.69137969907</v>
+        <v>46164.524713032406</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>278</v>
@@ -6751,11 +6751,11 @@
         <v>279</v>
       </c>
       <c r="B90" s="5">
-        <v>46162.79261844908</v>
+        <v>46162.62595178241</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46164.69134153935</v>
+        <v>46164.524674872686</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>190</v>
@@ -6804,11 +6804,11 @@
         <v>282</v>
       </c>
       <c r="B91" s="9">
-        <v>46162.7926247338</v>
+        <v>46162.62595806713</v>
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46164.69133898148</v>
+        <v>46164.524672314816</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>190</v>
@@ -6857,11 +6857,11 @@
         <v>283</v>
       </c>
       <c r="B92" s="5">
-        <v>46162.792630682874</v>
+        <v>46162.6259640162</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46164.69133623842</v>
+        <v>46164.52466957176</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>190</v>
@@ -6910,11 +6910,11 @@
         <v>285</v>
       </c>
       <c r="B93" s="9">
-        <v>46162.79263777778</v>
+        <v>46162.62597111111</v>
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46164.691332372684</v>
+        <v>46164.52466570602</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>190</v>
@@ -6963,11 +6963,11 @@
         <v>286</v>
       </c>
       <c r="B94" s="5">
-        <v>46162.79268604166</v>
+        <v>46162.626019375</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46164.6915004051</v>
+        <v>46164.524833738426</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>287</v>
@@ -7026,11 +7026,11 @@
         <v>288</v>
       </c>
       <c r="B95" s="9">
-        <v>46162.79269070602</v>
+        <v>46162.62602403935</v>
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46164.691474872685</v>
+        <v>46164.52480820601</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>190</v>
@@ -7079,11 +7079,11 @@
         <v>290</v>
       </c>
       <c r="B96" s="5">
-        <v>46162.79269707176</v>
+        <v>46162.626030405096</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46164.69147140047</v>
+        <v>46164.524804733795</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>190</v>
@@ -7132,11 +7132,11 @@
         <v>292</v>
       </c>
       <c r="B97" s="9">
-        <v>46162.792703576386</v>
+        <v>46162.62603690972</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46164.691468171295</v>
+        <v>46164.52480150463</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>190</v>
@@ -7185,11 +7185,11 @@
         <v>294</v>
       </c>
       <c r="B98" s="5">
-        <v>46162.79271046296</v>
+        <v>46162.62604379629</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46164.69146488426</v>
+        <v>46164.52479821759</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>190</v>
@@ -7238,11 +7238,11 @@
         <v>297</v>
       </c>
       <c r="B99" s="9">
-        <v>46162.792744861115</v>
+        <v>46162.626078194444</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46164.691619942125</v>
+        <v>46164.52495327547</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>298</v>
@@ -7301,11 +7301,11 @@
         <v>299</v>
       </c>
       <c r="B100" s="5">
-        <v>46162.79274982639</v>
+        <v>46162.62608315972</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46164.69158721065</v>
+        <v>46164.52492054398</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>190</v>
@@ -7354,11 +7354,11 @@
         <v>302</v>
       </c>
       <c r="B101" s="9">
-        <v>46162.79275559028</v>
+        <v>46162.626088923615</v>
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46164.69158380787</v>
+        <v>46164.5249171412</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>190</v>
@@ -7407,11 +7407,11 @@
         <v>303</v>
       </c>
       <c r="B102" s="5">
-        <v>46162.79276118056</v>
+        <v>46162.62609451389</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46164.69158106481</v>
+        <v>46164.52491439815</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>190</v>
@@ -7460,11 +7460,11 @@
         <v>305</v>
       </c>
       <c r="B103" s="9">
-        <v>46162.792767754625</v>
+        <v>46162.62610108797</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46164.69157646991</v>
+        <v>46164.52490980324</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>190</v>
@@ -7513,11 +7513,11 @@
         <v>307</v>
       </c>
       <c r="B104" s="5">
-        <v>46162.79285696759</v>
+        <v>46162.62619030093</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46164.69173954861</v>
+        <v>46164.525072881945</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>308</v>
@@ -7576,11 +7576,11 @@
         <v>309</v>
       </c>
       <c r="B105" s="9">
-        <v>46162.792862511575</v>
+        <v>46162.6261958449</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46164.69170866898</v>
+        <v>46164.525042002315</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>190</v>
@@ -7629,11 +7629,11 @@
         <v>311</v>
       </c>
       <c r="B106" s="5">
-        <v>46162.792868125005</v>
+        <v>46162.62620145833</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46164.69170596065</v>
+        <v>46164.52503929398</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>190</v>
@@ -7682,11 +7682,11 @@
         <v>313</v>
       </c>
       <c r="B107" s="9">
-        <v>46162.792873750004</v>
+        <v>46162.62620708333</v>
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46164.69170293982</v>
+        <v>46164.525036273146</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>190</v>
@@ -7735,11 +7735,11 @@
         <v>314</v>
       </c>
       <c r="B108" s="5">
-        <v>46162.7928793287</v>
+        <v>46162.62621266204</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46164.691698194445</v>
+        <v>46164.52503152778</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>190</v>
@@ -7788,11 +7788,11 @@
         <v>315</v>
       </c>
       <c r="B109" s="9">
-        <v>46162.792907696756</v>
+        <v>46162.62624103009</v>
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="9">
-        <v>46164.69185736111</v>
+        <v>46164.52519069445</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>316</v>
@@ -7849,11 +7849,11 @@
         <v>318</v>
       </c>
       <c r="B110" s="5">
-        <v>46162.79291289352</v>
+        <v>46162.62624622685</v>
       </c>
       <c r="C110" s="6"/>
       <c r="D110" s="5">
-        <v>46164.69182431713</v>
+        <v>46164.52515765047</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>190</v>
@@ -7902,11 +7902,11 @@
         <v>320</v>
       </c>
       <c r="B111" s="9">
-        <v>46162.79291758101</v>
+        <v>46162.626250914356</v>
       </c>
       <c r="C111" s="10"/>
       <c r="D111" s="9">
-        <v>46164.691821562505</v>
+        <v>46164.52515489583</v>
       </c>
       <c r="E111" s="10" t="s">
         <v>190</v>
@@ -7955,11 +7955,11 @@
         <v>321</v>
       </c>
       <c r="B112" s="5">
-        <v>46162.79292245371</v>
+        <v>46162.626255787036</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46164.691819155094</v>
+        <v>46164.52515248842</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>190</v>
@@ -8008,11 +8008,11 @@
         <v>322</v>
       </c>
       <c r="B113" s="9">
-        <v>46162.79293256944</v>
+        <v>46162.62626590278</v>
       </c>
       <c r="C113" s="10"/>
       <c r="D113" s="9">
-        <v>46164.69181509259</v>
+        <v>46164.52514842592</v>
       </c>
       <c r="E113" s="10" t="s">
         <v>190</v>
@@ -8061,11 +8061,11 @@
         <v>323</v>
       </c>
       <c r="B114" s="5">
-        <v>46162.7930040625</v>
+        <v>46162.626337395835</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46164.68546163195</v>
+        <v>46164.518794965275</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>324</v>
@@ -8108,11 +8108,11 @@
         <v>326</v>
       </c>
       <c r="B115" s="9">
-        <v>46162.79300806713</v>
+        <v>46162.626341400464</v>
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="9">
-        <v>46164.6922515162</v>
+        <v>46164.525584849536</v>
       </c>
       <c r="E115" s="10" t="s">
         <v>327</v>
@@ -8171,11 +8171,11 @@
         <v>331</v>
       </c>
       <c r="B116" s="5">
-        <v>46162.79301847222</v>
+        <v>46162.62635180556</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46164.69223148148</v>
+        <v>46164.525564814816</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>190</v>
@@ -8224,11 +8224,11 @@
         <v>333</v>
       </c>
       <c r="B117" s="9">
-        <v>46162.79302525463</v>
+        <v>46162.626358587964</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="9">
-        <v>46164.69222814815</v>
+        <v>46164.52556148148</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>190</v>
@@ -8277,11 +8277,11 @@
         <v>334</v>
       </c>
       <c r="B118" s="5">
-        <v>46162.79303010416</v>
+        <v>46162.6263634375</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46164.69222525463</v>
+        <v>46164.525558587964</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>190</v>
@@ -8330,11 +8330,11 @@
         <v>336</v>
       </c>
       <c r="B119" s="9">
-        <v>46162.79303482639</v>
+        <v>46162.62636815972</v>
       </c>
       <c r="C119" s="10"/>
       <c r="D119" s="9">
-        <v>46164.69222011574</v>
+        <v>46164.52555344907</v>
       </c>
       <c r="E119" s="10" t="s">
         <v>190</v>
@@ -8383,11 +8383,11 @@
         <v>337</v>
       </c>
       <c r="B120" s="5">
-        <v>46162.79306296296</v>
+        <v>46162.6263962963</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46164.692368958335</v>
+        <v>46164.52570229166</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>338</v>
@@ -8446,11 +8446,11 @@
         <v>339</v>
       </c>
       <c r="B121" s="9">
-        <v>46162.7930678125</v>
+        <v>46162.62640114583</v>
       </c>
       <c r="C121" s="10"/>
       <c r="D121" s="9">
-        <v>46164.692334189815</v>
+        <v>46164.52566752315</v>
       </c>
       <c r="E121" s="10" t="s">
         <v>190</v>
@@ -8499,11 +8499,11 @@
         <v>341</v>
       </c>
       <c r="B122" s="5">
-        <v>46162.793072280096</v>
+        <v>46162.626405613424</v>
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46164.6923315162</v>
+        <v>46164.52566484954</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>190</v>
@@ -8552,11 +8552,11 @@
         <v>342</v>
       </c>
       <c r="B123" s="9">
-        <v>46162.79307696759</v>
+        <v>46162.62641030093</v>
       </c>
       <c r="C123" s="10"/>
       <c r="D123" s="9">
-        <v>46164.69232880787</v>
+        <v>46164.525662141205</v>
       </c>
       <c r="E123" s="10" t="s">
         <v>190</v>
@@ -8605,11 +8605,11 @@
         <v>344</v>
       </c>
       <c r="B124" s="5">
-        <v>46162.79308175926</v>
+        <v>46162.62641509259</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46164.69232427083</v>
+        <v>46164.52565760417</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>190</v>
@@ -8658,11 +8658,11 @@
         <v>345</v>
       </c>
       <c r="B125" s="9">
-        <v>46162.79314625</v>
+        <v>46162.626479583334</v>
       </c>
       <c r="C125" s="10"/>
       <c r="D125" s="9">
-        <v>46164.69248696759</v>
+        <v>46164.52582030093</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>346</v>
@@ -8721,11 +8721,11 @@
         <v>347</v>
       </c>
       <c r="B126" s="5">
-        <v>46162.793151550926</v>
+        <v>46162.626484884255</v>
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46164.69246075231</v>
+        <v>46164.525794085646</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>190</v>
@@ -8774,11 +8774,11 @@
         <v>349</v>
       </c>
       <c r="B127" s="9">
-        <v>46162.79315885417</v>
+        <v>46162.6264921875</v>
       </c>
       <c r="C127" s="10"/>
       <c r="D127" s="9">
-        <v>46164.692458101854</v>
+        <v>46164.52579143518</v>
       </c>
       <c r="E127" s="10" t="s">
         <v>190</v>
@@ -8827,11 +8827,11 @@
         <v>350</v>
       </c>
       <c r="B128" s="5">
-        <v>46162.79316501158</v>
+        <v>46162.62649834491</v>
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46164.69245559028</v>
+        <v>46164.52578892361</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>190</v>
@@ -8880,11 +8880,11 @@
         <v>352</v>
       </c>
       <c r="B129" s="9">
-        <v>46162.79316986111</v>
+        <v>46162.62650319445</v>
       </c>
       <c r="C129" s="10"/>
       <c r="D129" s="9">
-        <v>46164.69245128472</v>
+        <v>46164.525784618054</v>
       </c>
       <c r="E129" s="10" t="s">
         <v>190</v>
@@ -8933,11 +8933,11 @@
         <v>354</v>
       </c>
       <c r="B130" s="5">
-        <v>46162.79319725695</v>
+        <v>46162.62653059028</v>
       </c>
       <c r="C130" s="6"/>
       <c r="D130" s="5">
-        <v>46164.69262644676</v>
+        <v>46164.52595978009</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>355</v>
@@ -8996,11 +8996,11 @@
         <v>357</v>
       </c>
       <c r="B131" s="9">
-        <v>46162.79320210648</v>
+        <v>46162.62653543982</v>
       </c>
       <c r="C131" s="10"/>
       <c r="D131" s="9">
-        <v>46164.692587303245</v>
+        <v>46164.52592063657</v>
       </c>
       <c r="E131" s="10" t="s">
         <v>190</v>
@@ -9049,11 +9049,11 @@
         <v>358</v>
       </c>
       <c r="B132" s="5">
-        <v>46162.793206111106</v>
+        <v>46162.62653944445</v>
       </c>
       <c r="C132" s="6"/>
       <c r="D132" s="5">
-        <v>46164.69258451389</v>
+        <v>46164.52591784722</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>190</v>
@@ -9102,11 +9102,11 @@
         <v>359</v>
       </c>
       <c r="B133" s="9">
-        <v>46162.7932099537</v>
+        <v>46162.62654328704</v>
       </c>
       <c r="C133" s="10"/>
       <c r="D133" s="9">
-        <v>46164.69258188657</v>
+        <v>46164.52591521991</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>190</v>
@@ -9155,11 +9155,11 @@
         <v>360</v>
       </c>
       <c r="B134" s="5">
-        <v>46162.79321400463</v>
+        <v>46162.62654733796</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46164.69257741898</v>
+        <v>46164.525910752316</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>190</v>
@@ -9208,11 +9208,11 @@
         <v>361</v>
       </c>
       <c r="B135" s="9">
-        <v>46162.79323766204</v>
+        <v>46162.62657099537</v>
       </c>
       <c r="C135" s="10"/>
       <c r="D135" s="9">
-        <v>46164.685922812496</v>
+        <v>46164.51925614583</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>362</v>
@@ -9255,11 +9255,11 @@
         <v>364</v>
       </c>
       <c r="B136" s="5">
-        <v>46162.79324063657</v>
+        <v>46162.62657396991</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46164.69269384259</v>
+        <v>46164.526027175925</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>365</v>
@@ -9318,11 +9318,11 @@
         <v>368</v>
       </c>
       <c r="B137" s="9">
-        <v>46162.79324528935</v>
+        <v>46162.62657862269</v>
       </c>
       <c r="C137" s="10"/>
       <c r="D137" s="9">
-        <v>46164.69273445602</v>
+        <v>46164.52606778935</v>
       </c>
       <c r="E137" s="10" t="s">
         <v>369</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-29 22:37 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
@@ -1771,13 +1771,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46162.79178179398</v>
+        <v>46162.62511512732</v>
       </c>
       <c r="C4" s="5">
-        <v>46183.58133199074</v>
+        <v>46183.414665324075</v>
       </c>
       <c r="D4" s="5">
-        <v>46183.58134738426</v>
+        <v>46183.41468071759</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1824,13 +1824,13 @@
         <v>28</v>
       </c>
       <c r="B5" s="9">
-        <v>46162.79189126157</v>
+        <v>46162.62522459491</v>
       </c>
       <c r="C5" s="9">
-        <v>46183.58129599537</v>
+        <v>46183.414629328705</v>
       </c>
       <c r="D5" s="9">
-        <v>46183.581316400465</v>
+        <v>46183.41464973379</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>29</v>
@@ -1889,13 +1889,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46162.79189434028</v>
+        <v>46162.62522767361</v>
       </c>
       <c r="C6" s="5">
-        <v>46183.58130109953</v>
+        <v>46183.41463443287</v>
       </c>
       <c r="D6" s="5">
-        <v>46183.58131646991</v>
+        <v>46183.41464980324</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1954,13 +1954,13 @@
         <v>36</v>
       </c>
       <c r="B7" s="9">
-        <v>46162.79190123842</v>
+        <v>46162.62523457176</v>
       </c>
       <c r="C7" s="9">
-        <v>46183.58131381945</v>
+        <v>46183.41464715278</v>
       </c>
       <c r="D7" s="9">
-        <v>46183.58133177084</v>
+        <v>46183.41466510417</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>37</v>
@@ -2019,13 +2019,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46162.791904513884</v>
+        <v>46162.62523784723</v>
       </c>
       <c r="C8" s="5">
-        <v>46183.581319641205</v>
+        <v>46183.414652974534</v>
       </c>
       <c r="D8" s="5">
-        <v>46183.58133340278</v>
+        <v>46183.41466673611</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2084,11 +2084,11 @@
         <v>43</v>
       </c>
       <c r="B9" s="9">
-        <v>46162.79178665509</v>
+        <v>46162.62511998843</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="9">
-        <v>46197.77681821759</v>
+        <v>46197.61015155092</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>44</v>
@@ -2133,13 +2133,13 @@
         <v>46</v>
       </c>
       <c r="B10" s="5">
-        <v>46162.7919078125</v>
+        <v>46162.62524114583</v>
       </c>
       <c r="C10" s="5">
-        <v>46197.659032407406</v>
+        <v>46197.49236574074</v>
       </c>
       <c r="D10" s="5">
-        <v>46197.776808263894</v>
+        <v>46197.61014159722</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>47</v>
@@ -2198,13 +2198,13 @@
         <v>53</v>
       </c>
       <c r="B11" s="9">
-        <v>46162.79191291667</v>
+        <v>46162.62524625</v>
       </c>
       <c r="C11" s="9">
-        <v>46197.660673125</v>
+        <v>46197.494006458335</v>
       </c>
       <c r="D11" s="9">
-        <v>46197.77680832176</v>
+        <v>46197.610141655096</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>54</v>
@@ -2263,13 +2263,13 @@
         <v>57</v>
       </c>
       <c r="B12" s="5">
-        <v>46162.791918055555</v>
+        <v>46162.62525138889</v>
       </c>
       <c r="C12" s="5">
-        <v>46197.66269631944</v>
+        <v>46197.49602965278</v>
       </c>
       <c r="D12" s="5">
-        <v>46197.776808344905</v>
+        <v>46197.61014167824</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>58</v>
@@ -2328,11 +2328,11 @@
         <v>61</v>
       </c>
       <c r="B13" s="9">
-        <v>46162.791791192125</v>
+        <v>46162.62512452547</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="9">
-        <v>46198.681430613426</v>
+        <v>46198.51476394676</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>62</v>
@@ -2375,13 +2375,13 @@
         <v>64</v>
       </c>
       <c r="B14" s="5">
-        <v>46162.79193019676</v>
+        <v>46162.62526353009</v>
       </c>
       <c r="C14" s="5">
-        <v>46198.68140460648</v>
+        <v>46198.51473793981</v>
       </c>
       <c r="D14" s="5">
-        <v>46198.68142037037</v>
+        <v>46198.514753703705</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>65</v>
@@ -2440,13 +2440,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="9">
-        <v>46162.7919353125</v>
+        <v>46162.62526864583</v>
       </c>
       <c r="C15" s="9">
-        <v>46198.68142288194</v>
+        <v>46198.51475621528</v>
       </c>
       <c r="D15" s="9">
-        <v>46198.68143896991</v>
+        <v>46198.51477230324</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>68</v>
@@ -2505,13 +2505,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46162.79194023148</v>
+        <v>46162.625273564816</v>
       </c>
       <c r="C16" s="5">
-        <v>46197.5874865625</v>
+        <v>46197.42081989584</v>
       </c>
       <c r="D16" s="5">
-        <v>46197.6606925</v>
+        <v>46197.49402583334</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2570,11 +2570,11 @@
         <v>74</v>
       </c>
       <c r="B17" s="9">
-        <v>46162.791945289355</v>
+        <v>46162.62527862268</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46198.78275258101</v>
+        <v>46198.61608591436</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>75</v>
@@ -2633,11 +2633,11 @@
         <v>80</v>
       </c>
       <c r="B18" s="5">
-        <v>46162.79194956018</v>
+        <v>46162.62528289352</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46198.78275320602</v>
+        <v>46198.61608653935</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>81</v>
@@ -2696,11 +2696,11 @@
         <v>83</v>
       </c>
       <c r="B19" s="9">
-        <v>46162.79195284723</v>
+        <v>46162.625286180555</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46198.782752604166</v>
+        <v>46198.6160859375</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>84</v>
@@ -2759,11 +2759,11 @@
         <v>86</v>
       </c>
       <c r="B20" s="5">
-        <v>46162.79195601852</v>
+        <v>46162.625289351854</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46198.78275268518</v>
+        <v>46198.61608601852</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>87</v>
@@ -2822,11 +2822,11 @@
         <v>89</v>
       </c>
       <c r="B21" s="9">
-        <v>46162.79179634259</v>
+        <v>46162.62512967593</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46198.685960648145</v>
+        <v>46198.51929398148</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>90</v>
@@ -2869,13 +2869,13 @@
         <v>92</v>
       </c>
       <c r="B22" s="5">
-        <v>46162.79196002315</v>
+        <v>46162.62529335648</v>
       </c>
       <c r="C22" s="5">
-        <v>46198.68595238426</v>
+        <v>46198.51928571759</v>
       </c>
       <c r="D22" s="5">
-        <v>46198.68596357639</v>
+        <v>46198.519296909726</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>93</v>
@@ -2934,13 +2934,13 @@
         <v>97</v>
       </c>
       <c r="B23" s="9">
-        <v>46162.791964375</v>
+        <v>46162.625297708335</v>
       </c>
       <c r="C23" s="9">
-        <v>46198.685906238425</v>
+        <v>46198.51923957176</v>
       </c>
       <c r="D23" s="9">
-        <v>46198.68590748843</v>
+        <v>46198.519240821755</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>98</v>
@@ -2995,13 +2995,13 @@
         <v>101</v>
       </c>
       <c r="B24" s="5">
-        <v>46162.79196883102</v>
+        <v>46162.62530216435</v>
       </c>
       <c r="C24" s="5">
-        <v>46198.68593903935</v>
+        <v>46198.51927237269</v>
       </c>
       <c r="D24" s="5">
-        <v>46198.6859406713</v>
+        <v>46198.51927400463</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>102</v>
@@ -3056,11 +3056,11 @@
         <v>104</v>
       </c>
       <c r="B25" s="9">
-        <v>46162.79197329861</v>
+        <v>46162.62530663195</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="9">
-        <v>46169.17544910879</v>
+        <v>46169.00878244213</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>105</v>
@@ -3119,11 +3119,11 @@
         <v>107</v>
       </c>
       <c r="B26" s="5">
-        <v>46162.791977500005</v>
+        <v>46162.62531083333</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46197.58749420139</v>
+        <v>46197.42082753472</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>108</v>
@@ -3178,11 +3178,11 @@
         <v>110</v>
       </c>
       <c r="B27" s="9">
-        <v>46162.79198199074</v>
+        <v>46162.62531532407</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="9">
-        <v>46168.172647141204</v>
+        <v>46168.00598047454</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>111</v>
@@ -3237,13 +3237,13 @@
         <v>113</v>
       </c>
       <c r="B28" s="5">
-        <v>46162.79198653935</v>
+        <v>46162.625319872684</v>
       </c>
       <c r="C28" s="5">
-        <v>46198.685692280094</v>
+        <v>46198.51902561342</v>
       </c>
       <c r="D28" s="5">
-        <v>46198.68573546296</v>
+        <v>46198.5190687963</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>114</v>
@@ -3302,13 +3302,13 @@
         <v>116</v>
       </c>
       <c r="B29" s="9">
-        <v>46162.79199082176</v>
+        <v>46162.62532415509</v>
       </c>
       <c r="C29" s="9">
-        <v>46198.68152349537</v>
+        <v>46198.514856828704</v>
       </c>
       <c r="D29" s="9">
-        <v>46198.68152484954</v>
+        <v>46198.51485818287</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>117</v>
@@ -3363,13 +3363,13 @@
         <v>119</v>
       </c>
       <c r="B30" s="5">
-        <v>46162.791995312495</v>
+        <v>46162.62532864584</v>
       </c>
       <c r="C30" s="5">
-        <v>46198.68567659722</v>
+        <v>46198.519009930555</v>
       </c>
       <c r="D30" s="5">
-        <v>46198.68567791667</v>
+        <v>46198.51901125</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>120</v>
@@ -3424,13 +3424,13 @@
         <v>122</v>
       </c>
       <c r="B31" s="9">
-        <v>46162.79199990741</v>
+        <v>46162.625333240736</v>
       </c>
       <c r="C31" s="9">
-        <v>46198.681561550926</v>
+        <v>46198.514894884254</v>
       </c>
       <c r="D31" s="9">
-        <v>46198.68156315973</v>
+        <v>46198.514896493056</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>123</v>
@@ -3485,11 +3485,11 @@
         <v>125</v>
       </c>
       <c r="B32" s="5">
-        <v>46162.792004421295</v>
+        <v>46162.62533775463</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46164.68978111111</v>
+        <v>46164.52311444444</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>126</v>
@@ -3548,11 +3548,11 @@
         <v>130</v>
       </c>
       <c r="B33" s="9">
-        <v>46162.79200878472</v>
+        <v>46162.62534211806</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="9">
-        <v>46164.68973819444</v>
+        <v>46164.52307152778</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>131</v>
@@ -3607,11 +3607,11 @@
         <v>133</v>
       </c>
       <c r="B34" s="5">
-        <v>46162.792013391205</v>
+        <v>46162.62534672454</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46164.68973515046</v>
+        <v>46164.523068483795</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>134</v>
@@ -3666,11 +3666,11 @@
         <v>136</v>
       </c>
       <c r="B35" s="9">
-        <v>46162.79201809027</v>
+        <v>46162.625351423616</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="9">
-        <v>46164.689874131946</v>
+        <v>46164.523207465274</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>137</v>
@@ -3729,11 +3729,11 @@
         <v>139</v>
       </c>
       <c r="B36" s="5">
-        <v>46162.79207501157</v>
+        <v>46162.6254083449</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46164.68984363426</v>
+        <v>46164.52317696759</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>82</v>
@@ -3782,11 +3782,11 @@
         <v>141</v>
       </c>
       <c r="B37" s="9">
-        <v>46162.79208025463</v>
+        <v>46162.625413587964</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="9">
-        <v>46164.68984076389</v>
+        <v>46164.52317409722</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>142</v>
@@ -3835,11 +3835,11 @@
         <v>144</v>
       </c>
       <c r="B38" s="5">
-        <v>46162.792085</v>
+        <v>46162.62541833334</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46164.69004553241</v>
+        <v>46164.52337886574</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>145</v>
@@ -3898,11 +3898,11 @@
         <v>149</v>
       </c>
       <c r="B39" s="9">
-        <v>46162.792089166665</v>
+        <v>46162.6254225</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="9">
-        <v>46164.68995886574</v>
+        <v>46164.523292199076</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>88</v>
@@ -3951,11 +3951,11 @@
         <v>151</v>
       </c>
       <c r="B40" s="5">
-        <v>46162.792093599535</v>
+        <v>46162.62542693287</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46164.68995591435</v>
+        <v>46164.523289247685</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>152</v>
@@ -4004,11 +4004,11 @@
         <v>154</v>
       </c>
       <c r="B41" s="9">
-        <v>46162.79210385417</v>
+        <v>46162.6254371875</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="9">
-        <v>46164.68998921296</v>
+        <v>46164.5233225463</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>155</v>
@@ -4057,11 +4057,11 @@
         <v>158</v>
       </c>
       <c r="B42" s="5">
-        <v>46162.79210730324</v>
+        <v>46162.62544063658</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46164.690100057865</v>
+        <v>46164.52343339121</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>159</v>
@@ -4120,11 +4120,11 @@
         <v>161</v>
       </c>
       <c r="B43" s="9">
-        <v>46162.792111180555</v>
+        <v>46162.62544451389</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="9">
-        <v>46164.690157951394</v>
+        <v>46164.52349128472</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>85</v>
@@ -4173,11 +4173,11 @@
         <v>163</v>
       </c>
       <c r="B44" s="5">
-        <v>46162.79211601852</v>
+        <v>46162.62544935185</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46164.69015534723</v>
+        <v>46164.523488680556</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>164</v>
@@ -4226,11 +4226,11 @@
         <v>166</v>
       </c>
       <c r="B45" s="9">
-        <v>46162.791800798615</v>
+        <v>46162.625134131944</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="9">
-        <v>46198.78268122685</v>
+        <v>46198.61601456019</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>167</v>
@@ -4275,13 +4275,13 @@
         <v>169</v>
       </c>
       <c r="B46" s="5">
-        <v>46162.79212121527</v>
+        <v>46162.625454548615</v>
       </c>
       <c r="C46" s="5">
-        <v>46197.680713587964</v>
+        <v>46197.51404692129</v>
       </c>
       <c r="D46" s="5">
-        <v>46197.68073020833</v>
+        <v>46197.51406354167</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>170</v>
@@ -4340,13 +4340,13 @@
         <v>174</v>
       </c>
       <c r="B47" s="9">
-        <v>46162.79212670139</v>
+        <v>46162.625460034724</v>
       </c>
       <c r="C47" s="9">
-        <v>46198.78266340277</v>
+        <v>46198.615996736116</v>
       </c>
       <c r="D47" s="9">
-        <v>46198.78268157407</v>
+        <v>46198.616014907406</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>175</v>
@@ -4405,13 +4405,13 @@
         <v>178</v>
       </c>
       <c r="B48" s="5">
-        <v>46162.792133090275</v>
+        <v>46162.62546642361</v>
       </c>
       <c r="C48" s="5">
-        <v>46198.78271623843</v>
+        <v>46198.61604957176</v>
       </c>
       <c r="D48" s="5">
-        <v>46198.7827322338</v>
+        <v>46198.61606556713</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>78</v>
@@ -4470,11 +4470,11 @@
         <v>182</v>
       </c>
       <c r="B49" s="9">
-        <v>46162.79214709491</v>
+        <v>46162.625480428236</v>
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="9">
-        <v>46164.69027550926</v>
+        <v>46164.52360884259</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>183</v>
@@ -4533,11 +4533,11 @@
         <v>187</v>
       </c>
       <c r="B50" s="5">
-        <v>46162.792150775465</v>
+        <v>46162.625484108794</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46164.69036847222</v>
+        <v>46164.523701805556</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>188</v>
@@ -4586,11 +4586,11 @@
         <v>190</v>
       </c>
       <c r="B51" s="9">
-        <v>46162.792154849536</v>
+        <v>46162.62548818287</v>
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="9">
-        <v>46164.69036586805</v>
+        <v>46164.52369920139</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>188</v>
@@ -4639,11 +4639,11 @@
         <v>191</v>
       </c>
       <c r="B52" s="5">
-        <v>46162.79215875</v>
+        <v>46162.62549208333</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46164.69036304398</v>
+        <v>46164.52369637731</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>188</v>
@@ -4692,11 +4692,11 @@
         <v>192</v>
       </c>
       <c r="B53" s="9">
-        <v>46162.79216164352</v>
+        <v>46162.62549497685</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="9">
-        <v>46164.690358935186</v>
+        <v>46164.523692268514</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>188</v>
@@ -4745,11 +4745,11 @@
         <v>193</v>
       </c>
       <c r="B54" s="5">
-        <v>46162.7922118287</v>
+        <v>46162.62554516204</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46164.66718020833</v>
+        <v>46164.500513541665</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4792,11 +4792,11 @@
         <v>196</v>
       </c>
       <c r="B55" s="9">
-        <v>46162.7922200926</v>
+        <v>46162.625553425925</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="9">
-        <v>46164.69048553241</v>
+        <v>46164.52381886574</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>197</v>
@@ -4855,11 +4855,11 @@
         <v>201</v>
       </c>
       <c r="B56" s="5">
-        <v>46162.792225625</v>
+        <v>46162.62555895833</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46164.69055459491</v>
+        <v>46164.52388792824</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>202</v>
@@ -4918,11 +4918,11 @@
         <v>205</v>
       </c>
       <c r="B57" s="9">
-        <v>46162.79223230324</v>
+        <v>46162.625565636576</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="9">
-        <v>46164.690482418984</v>
+        <v>46164.52381575231</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>206</v>
@@ -4981,11 +4981,11 @@
         <v>208</v>
       </c>
       <c r="B58" s="5">
-        <v>46162.79223737269</v>
+        <v>46162.62557070602</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46164.69055186343</v>
+        <v>46164.52388519676</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>209</v>
@@ -5044,11 +5044,11 @@
         <v>211</v>
       </c>
       <c r="B59" s="9">
-        <v>46162.7922424537</v>
+        <v>46162.62557578704</v>
       </c>
       <c r="C59" s="10"/>
       <c r="D59" s="9">
-        <v>46164.6904790625</v>
+        <v>46164.52381239583</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>212</v>
@@ -5107,11 +5107,11 @@
         <v>214</v>
       </c>
       <c r="B60" s="5">
-        <v>46162.792246909725</v>
+        <v>46162.62558024305</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46164.690549328705</v>
+        <v>46164.52388266203</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>213</v>
@@ -5170,11 +5170,11 @@
         <v>215</v>
       </c>
       <c r="B61" s="9">
-        <v>46162.79225168981</v>
+        <v>46162.62558502315</v>
       </c>
       <c r="C61" s="10"/>
       <c r="D61" s="9">
-        <v>46164.66898752315</v>
+        <v>46164.50232085648</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>216</v>
@@ -5217,11 +5217,11 @@
         <v>218</v>
       </c>
       <c r="B62" s="5">
-        <v>46162.792254479165</v>
+        <v>46162.6255878125</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46164.69072508102</v>
+        <v>46164.52405841435</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>219</v>
@@ -5280,11 +5280,11 @@
         <v>222</v>
       </c>
       <c r="B63" s="9">
-        <v>46162.79225922454</v>
+        <v>46162.62559255787</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46164.69068318287</v>
+        <v>46164.5240165162</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>188</v>
@@ -5333,11 +5333,11 @@
         <v>225</v>
       </c>
       <c r="B64" s="5">
-        <v>46162.792265578704</v>
+        <v>46162.62559891204</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46164.69068048611</v>
+        <v>46164.52401381945</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>188</v>
@@ -5386,11 +5386,11 @@
         <v>227</v>
       </c>
       <c r="B65" s="9">
-        <v>46162.79227201389</v>
+        <v>46162.62560534722</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="9">
-        <v>46164.69067753472</v>
+        <v>46164.52401086806</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>188</v>
@@ -5439,11 +5439,11 @@
         <v>230</v>
       </c>
       <c r="B66" s="5">
-        <v>46162.79227828704</v>
+        <v>46162.62561162037</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46164.69067336805</v>
+        <v>46164.52400670139</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>188</v>
@@ -5492,11 +5492,11 @@
         <v>231</v>
       </c>
       <c r="B67" s="9">
-        <v>46162.79232202546</v>
+        <v>46162.625655358795</v>
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="9">
-        <v>46164.69085144676</v>
+        <v>46164.52418478009</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>232</v>
@@ -5555,11 +5555,11 @@
         <v>233</v>
       </c>
       <c r="B68" s="5">
-        <v>46162.79232653935</v>
+        <v>46162.62565987269</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46198.782724606484</v>
+        <v>46198.61605793981</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>188</v>
@@ -5608,11 +5608,11 @@
         <v>236</v>
       </c>
       <c r="B69" s="9">
-        <v>46162.79233265047</v>
+        <v>46162.625665983796</v>
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46198.78272363426</v>
+        <v>46198.61605696759</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>188</v>
@@ -5661,11 +5661,11 @@
         <v>237</v>
       </c>
       <c r="B70" s="5">
-        <v>46162.79233820602</v>
+        <v>46162.625671539354</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46198.78273228009</v>
+        <v>46198.61606561343</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>188</v>
@@ -5714,11 +5714,11 @@
         <v>239</v>
       </c>
       <c r="B71" s="9">
-        <v>46162.79234384259</v>
+        <v>46162.62567717592</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46198.782732824075</v>
+        <v>46198.61606615741</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>188</v>
@@ -5767,11 +5767,11 @@
         <v>240</v>
       </c>
       <c r="B72" s="5">
-        <v>46162.79241414352</v>
+        <v>46162.62574747685</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46164.690976377315</v>
+        <v>46164.52430971064</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>241</v>
@@ -5830,11 +5830,11 @@
         <v>242</v>
       </c>
       <c r="B73" s="9">
-        <v>46162.79242041666</v>
+        <v>46162.62575375</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="9">
-        <v>46198.78273341435</v>
+        <v>46198.61606674769</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>188</v>
@@ -5883,11 +5883,11 @@
         <v>244</v>
       </c>
       <c r="B74" s="5">
-        <v>46162.79243321759</v>
+        <v>46162.625766550926</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46198.78272657408</v>
+        <v>46198.61605990741</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>188</v>
@@ -5936,11 +5936,11 @@
         <v>246</v>
       </c>
       <c r="B75" s="9">
-        <v>46162.79243956019</v>
+        <v>46162.625772893516</v>
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46198.78272707176</v>
+        <v>46198.6160604051</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>188</v>
@@ -5989,11 +5989,11 @@
         <v>248</v>
       </c>
       <c r="B76" s="5">
-        <v>46162.79244651621</v>
+        <v>46162.625779849535</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46198.78272166666</v>
+        <v>46198.616055</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>188</v>
@@ -6042,11 +6042,11 @@
         <v>249</v>
       </c>
       <c r="B77" s="9">
-        <v>46162.79247811342</v>
+        <v>46162.625811446764</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46164.670772627316</v>
+        <v>46164.504105960645</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>194</v>
@@ -6089,11 +6089,11 @@
         <v>251</v>
       </c>
       <c r="B78" s="5">
-        <v>46162.792481805554</v>
+        <v>46162.62581513889</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46171.19919608797</v>
+        <v>46171.032529421296</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>252</v>
@@ -6152,11 +6152,11 @@
         <v>254</v>
       </c>
       <c r="B79" s="9">
-        <v>46162.79248949074</v>
+        <v>46162.62582282408</v>
       </c>
       <c r="C79" s="10"/>
       <c r="D79" s="9">
-        <v>46198.68596158565</v>
+        <v>46198.51929491898</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>255</v>
@@ -6215,11 +6215,11 @@
         <v>257</v>
       </c>
       <c r="B80" s="5">
-        <v>46162.79249689815</v>
+        <v>46162.62583023148</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46198.68569559028</v>
+        <v>46198.51902892361</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>258</v>
@@ -6278,11 +6278,11 @@
         <v>259</v>
       </c>
       <c r="B81" s="9">
-        <v>46162.79250443287</v>
+        <v>46162.6258377662</v>
       </c>
       <c r="C81" s="10"/>
       <c r="D81" s="9">
-        <v>46164.69110619213</v>
+        <v>46164.52443952546</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>260</v>
@@ -6341,11 +6341,11 @@
         <v>262</v>
       </c>
       <c r="B82" s="5">
-        <v>46162.79250947917</v>
+        <v>46162.6258428125</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46164.68453591435</v>
+        <v>46164.517869247684</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>263</v>
@@ -6388,11 +6388,11 @@
         <v>265</v>
       </c>
       <c r="B83" s="9">
-        <v>46162.79251295139</v>
+        <v>46162.62584628472</v>
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46164.69124818287</v>
+        <v>46164.524581516205</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>266</v>
@@ -6451,11 +6451,11 @@
         <v>268</v>
       </c>
       <c r="B84" s="5">
-        <v>46162.79252873843</v>
+        <v>46162.625862071756</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46164.69121831018</v>
+        <v>46164.52455164352</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>188</v>
@@ -6504,11 +6504,11 @@
         <v>270</v>
       </c>
       <c r="B85" s="9">
-        <v>46162.792533518514</v>
+        <v>46162.62586685186</v>
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46164.6912157176</v>
+        <v>46164.524549050926</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>188</v>
@@ -6557,11 +6557,11 @@
         <v>271</v>
       </c>
       <c r="B86" s="5">
-        <v>46162.79253825231</v>
+        <v>46162.62587158565</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46164.69121336806</v>
+        <v>46164.52454670139</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>188</v>
@@ -6610,11 +6610,11 @@
         <v>273</v>
       </c>
       <c r="B87" s="9">
-        <v>46162.792543206015</v>
+        <v>46162.62587653935</v>
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46164.691209490746</v>
+        <v>46164.524542824074</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>188</v>
@@ -6663,11 +6663,11 @@
         <v>275</v>
       </c>
       <c r="B88" s="5">
-        <v>46162.792612743055</v>
+        <v>46162.62594607639</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46164.69137969907</v>
+        <v>46164.524713032406</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>276</v>
@@ -6726,11 +6726,11 @@
         <v>277</v>
       </c>
       <c r="B89" s="9">
-        <v>46162.79261844908</v>
+        <v>46162.62595178241</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46198.78274127315</v>
+        <v>46198.616074606485</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>188</v>
@@ -6779,11 +6779,11 @@
         <v>280</v>
       </c>
       <c r="B90" s="5">
-        <v>46162.7926247338</v>
+        <v>46162.62595806713</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46198.782722233795</v>
+        <v>46198.61605556713</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>188</v>
@@ -6832,11 +6832,11 @@
         <v>281</v>
       </c>
       <c r="B91" s="9">
-        <v>46162.792630682874</v>
+        <v>46162.6259640162</v>
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46198.78272511574</v>
+        <v>46198.61605844907</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>188</v>
@@ -6885,11 +6885,11 @@
         <v>283</v>
       </c>
       <c r="B92" s="5">
-        <v>46162.79263777778</v>
+        <v>46162.62597111111</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46198.782724108794</v>
+        <v>46198.61605744213</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>188</v>
@@ -6938,11 +6938,11 @@
         <v>284</v>
       </c>
       <c r="B93" s="9">
-        <v>46162.79268604166</v>
+        <v>46162.626019375</v>
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46164.6915004051</v>
+        <v>46164.524833738426</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>285</v>
@@ -7001,11 +7001,11 @@
         <v>286</v>
       </c>
       <c r="B94" s="5">
-        <v>46162.79269070602</v>
+        <v>46162.62602403935</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46198.78272271991</v>
+        <v>46198.616056053244</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>188</v>
@@ -7054,11 +7054,11 @@
         <v>288</v>
       </c>
       <c r="B95" s="9">
-        <v>46162.79269707176</v>
+        <v>46162.626030405096</v>
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46198.78272560185</v>
+        <v>46198.616058935186</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>188</v>
@@ -7107,11 +7107,11 @@
         <v>290</v>
       </c>
       <c r="B96" s="5">
-        <v>46162.792703576386</v>
+        <v>46162.62603690972</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46198.78273373842</v>
+        <v>46198.61606707176</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>188</v>
@@ -7160,11 +7160,11 @@
         <v>292</v>
       </c>
       <c r="B97" s="9">
-        <v>46162.79271046296</v>
+        <v>46162.62604379629</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46198.78272606482</v>
+        <v>46198.61605939815</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>188</v>
@@ -7213,11 +7213,11 @@
         <v>295</v>
       </c>
       <c r="B98" s="5">
-        <v>46162.792744861115</v>
+        <v>46162.626078194444</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46164.691619942125</v>
+        <v>46164.52495327547</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>296</v>
@@ -7276,11 +7276,11 @@
         <v>297</v>
       </c>
       <c r="B99" s="9">
-        <v>46162.79274982639</v>
+        <v>46162.62608315972</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46198.78272754629</v>
+        <v>46198.616060879634</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>188</v>
@@ -7329,11 +7329,11 @@
         <v>300</v>
       </c>
       <c r="B100" s="5">
-        <v>46162.79275559028</v>
+        <v>46162.626088923615</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46198.78272310185</v>
+        <v>46198.61605643519</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>188</v>
@@ -7382,11 +7382,11 @@
         <v>301</v>
       </c>
       <c r="B101" s="9">
-        <v>46162.79276118056</v>
+        <v>46162.62609451389</v>
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46198.782727893515</v>
+        <v>46198.61606122685</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>188</v>
@@ -7435,11 +7435,11 @@
         <v>303</v>
       </c>
       <c r="B102" s="5">
-        <v>46162.792767754625</v>
+        <v>46162.62610108797</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46198.782728391205</v>
+        <v>46198.61606172453</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>188</v>
@@ -7488,11 +7488,11 @@
         <v>305</v>
       </c>
       <c r="B103" s="9">
-        <v>46162.79285696759</v>
+        <v>46162.62619030093</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46164.69173954861</v>
+        <v>46164.525072881945</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>306</v>
@@ -7551,11 +7551,11 @@
         <v>307</v>
       </c>
       <c r="B104" s="5">
-        <v>46162.792862511575</v>
+        <v>46162.6261958449</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46164.69170866898</v>
+        <v>46164.525042002315</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>188</v>
@@ -7604,11 +7604,11 @@
         <v>309</v>
       </c>
       <c r="B105" s="9">
-        <v>46162.792868125005</v>
+        <v>46162.62620145833</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46164.69170596065</v>
+        <v>46164.52503929398</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>188</v>
@@ -7657,11 +7657,11 @@
         <v>311</v>
       </c>
       <c r="B106" s="5">
-        <v>46162.792873750004</v>
+        <v>46162.62620708333</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46164.69170293982</v>
+        <v>46164.525036273146</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>188</v>
@@ -7710,11 +7710,11 @@
         <v>312</v>
       </c>
       <c r="B107" s="9">
-        <v>46162.7928793287</v>
+        <v>46162.62621266204</v>
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46164.691698194445</v>
+        <v>46164.52503152778</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>188</v>
@@ -7763,11 +7763,11 @@
         <v>313</v>
       </c>
       <c r="B108" s="5">
-        <v>46162.792907696756</v>
+        <v>46162.62624103009</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46164.69185736111</v>
+        <v>46164.52519069445</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>314</v>
@@ -7824,11 +7824,11 @@
         <v>316</v>
       </c>
       <c r="B109" s="9">
-        <v>46162.79291289352</v>
+        <v>46162.62624622685</v>
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="9">
-        <v>46164.69182431713</v>
+        <v>46164.52515765047</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>188</v>
@@ -7877,11 +7877,11 @@
         <v>318</v>
       </c>
       <c r="B110" s="5">
-        <v>46162.79291758101</v>
+        <v>46162.626250914356</v>
       </c>
       <c r="C110" s="6"/>
       <c r="D110" s="5">
-        <v>46164.691821562505</v>
+        <v>46164.52515489583</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>188</v>
@@ -7930,11 +7930,11 @@
         <v>319</v>
       </c>
       <c r="B111" s="9">
-        <v>46162.79292245371</v>
+        <v>46162.626255787036</v>
       </c>
       <c r="C111" s="10"/>
       <c r="D111" s="9">
-        <v>46164.691819155094</v>
+        <v>46164.52515248842</v>
       </c>
       <c r="E111" s="10" t="s">
         <v>188</v>
@@ -7983,11 +7983,11 @@
         <v>320</v>
       </c>
       <c r="B112" s="5">
-        <v>46162.79293256944</v>
+        <v>46162.62626590278</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46164.69181509259</v>
+        <v>46164.52514842592</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>188</v>
@@ -8036,11 +8036,11 @@
         <v>321</v>
       </c>
       <c r="B113" s="9">
-        <v>46162.7930040625</v>
+        <v>46162.626337395835</v>
       </c>
       <c r="C113" s="10"/>
       <c r="D113" s="9">
-        <v>46164.68546163195</v>
+        <v>46164.518794965275</v>
       </c>
       <c r="E113" s="10" t="s">
         <v>322</v>
@@ -8083,11 +8083,11 @@
         <v>324</v>
       </c>
       <c r="B114" s="5">
-        <v>46162.79300806713</v>
+        <v>46162.626341400464</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46164.6922515162</v>
+        <v>46164.525584849536</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>325</v>
@@ -8146,11 +8146,11 @@
         <v>329</v>
       </c>
       <c r="B115" s="9">
-        <v>46162.79301847222</v>
+        <v>46162.62635180556</v>
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="9">
-        <v>46164.69223148148</v>
+        <v>46164.525564814816</v>
       </c>
       <c r="E115" s="10" t="s">
         <v>188</v>
@@ -8199,11 +8199,11 @@
         <v>331</v>
       </c>
       <c r="B116" s="5">
-        <v>46162.79302525463</v>
+        <v>46162.626358587964</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46164.69222814815</v>
+        <v>46164.52556148148</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>188</v>
@@ -8252,11 +8252,11 @@
         <v>332</v>
       </c>
       <c r="B117" s="9">
-        <v>46162.79303010416</v>
+        <v>46162.6263634375</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="9">
-        <v>46164.69222525463</v>
+        <v>46164.525558587964</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>188</v>
@@ -8305,11 +8305,11 @@
         <v>334</v>
       </c>
       <c r="B118" s="5">
-        <v>46162.79303482639</v>
+        <v>46162.62636815972</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46164.69222011574</v>
+        <v>46164.52555344907</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>188</v>
@@ -8358,11 +8358,11 @@
         <v>335</v>
       </c>
       <c r="B119" s="9">
-        <v>46162.79306296296</v>
+        <v>46162.6263962963</v>
       </c>
       <c r="C119" s="10"/>
       <c r="D119" s="9">
-        <v>46164.692368958335</v>
+        <v>46164.52570229166</v>
       </c>
       <c r="E119" s="10" t="s">
         <v>336</v>
@@ -8421,11 +8421,11 @@
         <v>337</v>
       </c>
       <c r="B120" s="5">
-        <v>46162.7930678125</v>
+        <v>46162.62640114583</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46164.692334189815</v>
+        <v>46164.52566752315</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>188</v>
@@ -8474,11 +8474,11 @@
         <v>339</v>
       </c>
       <c r="B121" s="9">
-        <v>46162.793072280096</v>
+        <v>46162.626405613424</v>
       </c>
       <c r="C121" s="10"/>
       <c r="D121" s="9">
-        <v>46164.6923315162</v>
+        <v>46164.52566484954</v>
       </c>
       <c r="E121" s="10" t="s">
         <v>188</v>
@@ -8527,11 +8527,11 @@
         <v>340</v>
       </c>
       <c r="B122" s="5">
-        <v>46162.79307696759</v>
+        <v>46162.62641030093</v>
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46164.69232880787</v>
+        <v>46164.525662141205</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>188</v>
@@ -8580,11 +8580,11 @@
         <v>342</v>
       </c>
       <c r="B123" s="9">
-        <v>46162.79308175926</v>
+        <v>46162.62641509259</v>
       </c>
       <c r="C123" s="10"/>
       <c r="D123" s="9">
-        <v>46164.69232427083</v>
+        <v>46164.52565760417</v>
       </c>
       <c r="E123" s="10" t="s">
         <v>188</v>
@@ -8633,11 +8633,11 @@
         <v>343</v>
       </c>
       <c r="B124" s="5">
-        <v>46162.79314625</v>
+        <v>46162.626479583334</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46164.69248696759</v>
+        <v>46164.52582030093</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>344</v>
@@ -8696,11 +8696,11 @@
         <v>345</v>
       </c>
       <c r="B125" s="9">
-        <v>46162.793151550926</v>
+        <v>46162.626484884255</v>
       </c>
       <c r="C125" s="10"/>
       <c r="D125" s="9">
-        <v>46164.69246075231</v>
+        <v>46164.525794085646</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>188</v>
@@ -8749,11 +8749,11 @@
         <v>347</v>
       </c>
       <c r="B126" s="5">
-        <v>46162.79315885417</v>
+        <v>46162.6264921875</v>
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46164.692458101854</v>
+        <v>46164.52579143518</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>188</v>
@@ -8802,11 +8802,11 @@
         <v>348</v>
       </c>
       <c r="B127" s="9">
-        <v>46162.79316501158</v>
+        <v>46162.62649834491</v>
       </c>
       <c r="C127" s="10"/>
       <c r="D127" s="9">
-        <v>46164.69245559028</v>
+        <v>46164.52578892361</v>
       </c>
       <c r="E127" s="10" t="s">
         <v>188</v>
@@ -8855,11 +8855,11 @@
         <v>350</v>
       </c>
       <c r="B128" s="5">
-        <v>46162.79316986111</v>
+        <v>46162.62650319445</v>
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46164.69245128472</v>
+        <v>46164.525784618054</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>188</v>
@@ -8908,11 +8908,11 @@
         <v>352</v>
       </c>
       <c r="B129" s="9">
-        <v>46162.79319725695</v>
+        <v>46162.62653059028</v>
       </c>
       <c r="C129" s="10"/>
       <c r="D129" s="9">
-        <v>46164.69262644676</v>
+        <v>46164.52595978009</v>
       </c>
       <c r="E129" s="10" t="s">
         <v>353</v>
@@ -8971,11 +8971,11 @@
         <v>355</v>
       </c>
       <c r="B130" s="5">
-        <v>46162.79320210648</v>
+        <v>46162.62653543982</v>
       </c>
       <c r="C130" s="6"/>
       <c r="D130" s="5">
-        <v>46164.692587303245</v>
+        <v>46164.52592063657</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>188</v>
@@ -9024,11 +9024,11 @@
         <v>356</v>
       </c>
       <c r="B131" s="9">
-        <v>46162.793206111106</v>
+        <v>46162.62653944445</v>
       </c>
       <c r="C131" s="10"/>
       <c r="D131" s="9">
-        <v>46164.69258451389</v>
+        <v>46164.52591784722</v>
       </c>
       <c r="E131" s="10" t="s">
         <v>188</v>
@@ -9077,11 +9077,11 @@
         <v>357</v>
       </c>
       <c r="B132" s="5">
-        <v>46162.7932099537</v>
+        <v>46162.62654328704</v>
       </c>
       <c r="C132" s="6"/>
       <c r="D132" s="5">
-        <v>46164.69258188657</v>
+        <v>46164.52591521991</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>188</v>
@@ -9130,11 +9130,11 @@
         <v>358</v>
       </c>
       <c r="B133" s="9">
-        <v>46162.79321400463</v>
+        <v>46162.62654733796</v>
       </c>
       <c r="C133" s="10"/>
       <c r="D133" s="9">
-        <v>46164.69257741898</v>
+        <v>46164.525910752316</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>188</v>
@@ -9183,11 +9183,11 @@
         <v>359</v>
       </c>
       <c r="B134" s="5">
-        <v>46162.79323766204</v>
+        <v>46162.62657099537</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46164.685922812496</v>
+        <v>46164.51925614583</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>360</v>
@@ -9230,11 +9230,11 @@
         <v>362</v>
       </c>
       <c r="B135" s="9">
-        <v>46162.79324063657</v>
+        <v>46162.62657396991</v>
       </c>
       <c r="C135" s="10"/>
       <c r="D135" s="9">
-        <v>46164.69269384259</v>
+        <v>46164.526027175925</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>363</v>
@@ -9293,11 +9293,11 @@
         <v>366</v>
       </c>
       <c r="B136" s="5">
-        <v>46162.79324528935</v>
+        <v>46162.62657862269</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46197.77680827546</v>
+        <v>46197.61014160879</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>367</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-29 23:11 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
@@ -1771,13 +1771,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46162.62511512732</v>
+        <v>46162.79178179398</v>
       </c>
       <c r="C4" s="5">
-        <v>46183.414665324075</v>
+        <v>46183.58133199074</v>
       </c>
       <c r="D4" s="5">
-        <v>46183.41468071759</v>
+        <v>46183.58134738426</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1824,13 +1824,13 @@
         <v>28</v>
       </c>
       <c r="B5" s="9">
-        <v>46162.62522459491</v>
+        <v>46162.79189126157</v>
       </c>
       <c r="C5" s="9">
-        <v>46183.414629328705</v>
+        <v>46183.58129599537</v>
       </c>
       <c r="D5" s="9">
-        <v>46183.41464973379</v>
+        <v>46183.581316400465</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>29</v>
@@ -1889,13 +1889,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46162.62522767361</v>
+        <v>46162.79189434028</v>
       </c>
       <c r="C6" s="5">
-        <v>46183.41463443287</v>
+        <v>46183.58130109953</v>
       </c>
       <c r="D6" s="5">
-        <v>46183.41464980324</v>
+        <v>46183.58131646991</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1954,13 +1954,13 @@
         <v>36</v>
       </c>
       <c r="B7" s="9">
-        <v>46162.62523457176</v>
+        <v>46162.79190123842</v>
       </c>
       <c r="C7" s="9">
-        <v>46183.41464715278</v>
+        <v>46183.58131381945</v>
       </c>
       <c r="D7" s="9">
-        <v>46183.41466510417</v>
+        <v>46183.58133177084</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>37</v>
@@ -2019,13 +2019,13 @@
         <v>40</v>
       </c>
       <c r="B8" s="5">
-        <v>46162.62523784723</v>
+        <v>46162.791904513884</v>
       </c>
       <c r="C8" s="5">
-        <v>46183.414652974534</v>
+        <v>46183.581319641205</v>
       </c>
       <c r="D8" s="5">
-        <v>46183.41466673611</v>
+        <v>46183.58133340278</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>41</v>
@@ -2084,11 +2084,11 @@
         <v>43</v>
       </c>
       <c r="B9" s="9">
-        <v>46162.62511998843</v>
+        <v>46162.79178665509</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="9">
-        <v>46197.61015155092</v>
+        <v>46197.77681821759</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>44</v>
@@ -2133,13 +2133,13 @@
         <v>46</v>
       </c>
       <c r="B10" s="5">
-        <v>46162.62524114583</v>
+        <v>46162.7919078125</v>
       </c>
       <c r="C10" s="5">
-        <v>46197.49236574074</v>
+        <v>46197.659032407406</v>
       </c>
       <c r="D10" s="5">
-        <v>46197.61014159722</v>
+        <v>46197.776808263894</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>47</v>
@@ -2198,13 +2198,13 @@
         <v>53</v>
       </c>
       <c r="B11" s="9">
-        <v>46162.62524625</v>
+        <v>46162.79191291667</v>
       </c>
       <c r="C11" s="9">
-        <v>46197.494006458335</v>
+        <v>46197.660673125</v>
       </c>
       <c r="D11" s="9">
-        <v>46197.610141655096</v>
+        <v>46197.77680832176</v>
       </c>
       <c r="E11" s="10" t="s">
         <v>54</v>
@@ -2263,13 +2263,13 @@
         <v>57</v>
       </c>
       <c r="B12" s="5">
-        <v>46162.62525138889</v>
+        <v>46162.791918055555</v>
       </c>
       <c r="C12" s="5">
-        <v>46197.49602965278</v>
+        <v>46197.66269631944</v>
       </c>
       <c r="D12" s="5">
-        <v>46197.61014167824</v>
+        <v>46197.776808344905</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>58</v>
@@ -2328,11 +2328,11 @@
         <v>61</v>
       </c>
       <c r="B13" s="9">
-        <v>46162.62512452547</v>
+        <v>46162.791791192125</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="9">
-        <v>46198.51476394676</v>
+        <v>46198.681430613426</v>
       </c>
       <c r="E13" s="10" t="s">
         <v>62</v>
@@ -2375,13 +2375,13 @@
         <v>64</v>
       </c>
       <c r="B14" s="5">
-        <v>46162.62526353009</v>
+        <v>46162.79193019676</v>
       </c>
       <c r="C14" s="5">
-        <v>46198.51473793981</v>
+        <v>46198.68140460648</v>
       </c>
       <c r="D14" s="5">
-        <v>46198.514753703705</v>
+        <v>46198.68142037037</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>65</v>
@@ -2440,13 +2440,13 @@
         <v>67</v>
       </c>
       <c r="B15" s="9">
-        <v>46162.62526864583</v>
+        <v>46162.7919353125</v>
       </c>
       <c r="C15" s="9">
-        <v>46198.51475621528</v>
+        <v>46198.68142288194</v>
       </c>
       <c r="D15" s="9">
-        <v>46198.51477230324</v>
+        <v>46198.68143896991</v>
       </c>
       <c r="E15" s="10" t="s">
         <v>68</v>
@@ -2505,13 +2505,13 @@
         <v>70</v>
       </c>
       <c r="B16" s="5">
-        <v>46162.625273564816</v>
+        <v>46162.79194023148</v>
       </c>
       <c r="C16" s="5">
-        <v>46197.42081989584</v>
+        <v>46197.5874865625</v>
       </c>
       <c r="D16" s="5">
-        <v>46197.49402583334</v>
+        <v>46197.6606925</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>71</v>
@@ -2570,11 +2570,11 @@
         <v>74</v>
       </c>
       <c r="B17" s="9">
-        <v>46162.62527862268</v>
+        <v>46162.791945289355</v>
       </c>
       <c r="C17" s="10"/>
       <c r="D17" s="9">
-        <v>46198.61608591436</v>
+        <v>46198.78275258101</v>
       </c>
       <c r="E17" s="10" t="s">
         <v>75</v>
@@ -2633,11 +2633,11 @@
         <v>80</v>
       </c>
       <c r="B18" s="5">
-        <v>46162.62528289352</v>
+        <v>46162.79194956018</v>
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46198.61608653935</v>
+        <v>46198.78275320602</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>81</v>
@@ -2696,11 +2696,11 @@
         <v>83</v>
       </c>
       <c r="B19" s="9">
-        <v>46162.625286180555</v>
+        <v>46162.79195284723</v>
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46198.6160859375</v>
+        <v>46198.782752604166</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>84</v>
@@ -2759,11 +2759,11 @@
         <v>86</v>
       </c>
       <c r="B20" s="5">
-        <v>46162.625289351854</v>
+        <v>46162.79195601852</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="5">
-        <v>46198.61608601852</v>
+        <v>46198.78275268518</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>87</v>
@@ -2822,11 +2822,11 @@
         <v>89</v>
       </c>
       <c r="B21" s="9">
-        <v>46162.62512967593</v>
+        <v>46162.79179634259</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="9">
-        <v>46198.51929398148</v>
+        <v>46198.685960648145</v>
       </c>
       <c r="E21" s="10" t="s">
         <v>90</v>
@@ -2869,13 +2869,13 @@
         <v>92</v>
       </c>
       <c r="B22" s="5">
-        <v>46162.62529335648</v>
+        <v>46162.79196002315</v>
       </c>
       <c r="C22" s="5">
-        <v>46198.51928571759</v>
+        <v>46198.68595238426</v>
       </c>
       <c r="D22" s="5">
-        <v>46198.519296909726</v>
+        <v>46198.68596357639</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>93</v>
@@ -2934,13 +2934,13 @@
         <v>97</v>
       </c>
       <c r="B23" s="9">
-        <v>46162.625297708335</v>
+        <v>46162.791964375</v>
       </c>
       <c r="C23" s="9">
-        <v>46198.51923957176</v>
+        <v>46198.685906238425</v>
       </c>
       <c r="D23" s="9">
-        <v>46198.519240821755</v>
+        <v>46198.68590748843</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>98</v>
@@ -2995,13 +2995,13 @@
         <v>101</v>
       </c>
       <c r="B24" s="5">
-        <v>46162.62530216435</v>
+        <v>46162.79196883102</v>
       </c>
       <c r="C24" s="5">
-        <v>46198.51927237269</v>
+        <v>46198.68593903935</v>
       </c>
       <c r="D24" s="5">
-        <v>46198.51927400463</v>
+        <v>46198.6859406713</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>102</v>
@@ -3056,11 +3056,11 @@
         <v>104</v>
       </c>
       <c r="B25" s="9">
-        <v>46162.62530663195</v>
+        <v>46162.79197329861</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="9">
-        <v>46169.00878244213</v>
+        <v>46169.17544910879</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>105</v>
@@ -3119,11 +3119,11 @@
         <v>107</v>
       </c>
       <c r="B26" s="5">
-        <v>46162.62531083333</v>
+        <v>46162.791977500005</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="5">
-        <v>46197.42082753472</v>
+        <v>46197.58749420139</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>108</v>
@@ -3178,11 +3178,11 @@
         <v>110</v>
       </c>
       <c r="B27" s="9">
-        <v>46162.62531532407</v>
+        <v>46162.79198199074</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="9">
-        <v>46168.00598047454</v>
+        <v>46168.172647141204</v>
       </c>
       <c r="E27" s="10" t="s">
         <v>111</v>
@@ -3237,13 +3237,13 @@
         <v>113</v>
       </c>
       <c r="B28" s="5">
-        <v>46162.625319872684</v>
+        <v>46162.79198653935</v>
       </c>
       <c r="C28" s="5">
-        <v>46198.51902561342</v>
+        <v>46198.685692280094</v>
       </c>
       <c r="D28" s="5">
-        <v>46198.5190687963</v>
+        <v>46198.68573546296</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>114</v>
@@ -3302,13 +3302,13 @@
         <v>116</v>
       </c>
       <c r="B29" s="9">
-        <v>46162.62532415509</v>
+        <v>46162.79199082176</v>
       </c>
       <c r="C29" s="9">
-        <v>46198.514856828704</v>
+        <v>46198.68152349537</v>
       </c>
       <c r="D29" s="9">
-        <v>46198.51485818287</v>
+        <v>46198.68152484954</v>
       </c>
       <c r="E29" s="10" t="s">
         <v>117</v>
@@ -3363,13 +3363,13 @@
         <v>119</v>
       </c>
       <c r="B30" s="5">
-        <v>46162.62532864584</v>
+        <v>46162.791995312495</v>
       </c>
       <c r="C30" s="5">
-        <v>46198.519009930555</v>
+        <v>46198.68567659722</v>
       </c>
       <c r="D30" s="5">
-        <v>46198.51901125</v>
+        <v>46198.68567791667</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>120</v>
@@ -3424,13 +3424,13 @@
         <v>122</v>
       </c>
       <c r="B31" s="9">
-        <v>46162.625333240736</v>
+        <v>46162.79199990741</v>
       </c>
       <c r="C31" s="9">
-        <v>46198.514894884254</v>
+        <v>46198.681561550926</v>
       </c>
       <c r="D31" s="9">
-        <v>46198.514896493056</v>
+        <v>46198.68156315973</v>
       </c>
       <c r="E31" s="10" t="s">
         <v>123</v>
@@ -3485,11 +3485,11 @@
         <v>125</v>
       </c>
       <c r="B32" s="5">
-        <v>46162.62533775463</v>
+        <v>46162.792004421295</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="5">
-        <v>46164.52311444444</v>
+        <v>46164.68978111111</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>126</v>
@@ -3548,11 +3548,11 @@
         <v>130</v>
       </c>
       <c r="B33" s="9">
-        <v>46162.62534211806</v>
+        <v>46162.79200878472</v>
       </c>
       <c r="C33" s="10"/>
       <c r="D33" s="9">
-        <v>46164.52307152778</v>
+        <v>46164.68973819444</v>
       </c>
       <c r="E33" s="10" t="s">
         <v>131</v>
@@ -3607,11 +3607,11 @@
         <v>133</v>
       </c>
       <c r="B34" s="5">
-        <v>46162.62534672454</v>
+        <v>46162.792013391205</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="5">
-        <v>46164.523068483795</v>
+        <v>46164.68973515046</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>134</v>
@@ -3666,11 +3666,11 @@
         <v>136</v>
       </c>
       <c r="B35" s="9">
-        <v>46162.625351423616</v>
+        <v>46162.79201809027</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="9">
-        <v>46164.523207465274</v>
+        <v>46164.689874131946</v>
       </c>
       <c r="E35" s="10" t="s">
         <v>137</v>
@@ -3729,11 +3729,11 @@
         <v>139</v>
       </c>
       <c r="B36" s="5">
-        <v>46162.6254083449</v>
+        <v>46162.79207501157</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46164.52317696759</v>
+        <v>46164.68984363426</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>82</v>
@@ -3782,11 +3782,11 @@
         <v>141</v>
       </c>
       <c r="B37" s="9">
-        <v>46162.625413587964</v>
+        <v>46162.79208025463</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="9">
-        <v>46164.52317409722</v>
+        <v>46164.68984076389</v>
       </c>
       <c r="E37" s="10" t="s">
         <v>142</v>
@@ -3835,11 +3835,11 @@
         <v>144</v>
       </c>
       <c r="B38" s="5">
-        <v>46162.62541833334</v>
+        <v>46162.792085</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46164.52337886574</v>
+        <v>46164.69004553241</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>145</v>
@@ -3898,11 +3898,11 @@
         <v>149</v>
       </c>
       <c r="B39" s="9">
-        <v>46162.6254225</v>
+        <v>46162.792089166665</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="9">
-        <v>46164.523292199076</v>
+        <v>46164.68995886574</v>
       </c>
       <c r="E39" s="10" t="s">
         <v>88</v>
@@ -3951,11 +3951,11 @@
         <v>151</v>
       </c>
       <c r="B40" s="5">
-        <v>46162.62542693287</v>
+        <v>46162.792093599535</v>
       </c>
       <c r="C40" s="6"/>
       <c r="D40" s="5">
-        <v>46164.523289247685</v>
+        <v>46164.68995591435</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>152</v>
@@ -4004,11 +4004,11 @@
         <v>154</v>
       </c>
       <c r="B41" s="9">
-        <v>46162.6254371875</v>
+        <v>46162.79210385417</v>
       </c>
       <c r="C41" s="10"/>
       <c r="D41" s="9">
-        <v>46164.5233225463</v>
+        <v>46164.68998921296</v>
       </c>
       <c r="E41" s="10" t="s">
         <v>155</v>
@@ -4057,11 +4057,11 @@
         <v>158</v>
       </c>
       <c r="B42" s="5">
-        <v>46162.62544063658</v>
+        <v>46162.79210730324</v>
       </c>
       <c r="C42" s="6"/>
       <c r="D42" s="5">
-        <v>46164.52343339121</v>
+        <v>46164.690100057865</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>159</v>
@@ -4120,11 +4120,11 @@
         <v>161</v>
       </c>
       <c r="B43" s="9">
-        <v>46162.62544451389</v>
+        <v>46162.792111180555</v>
       </c>
       <c r="C43" s="10"/>
       <c r="D43" s="9">
-        <v>46164.52349128472</v>
+        <v>46164.690157951394</v>
       </c>
       <c r="E43" s="10" t="s">
         <v>85</v>
@@ -4173,11 +4173,11 @@
         <v>163</v>
       </c>
       <c r="B44" s="5">
-        <v>46162.62544935185</v>
+        <v>46162.79211601852</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="5">
-        <v>46164.523488680556</v>
+        <v>46164.69015534723</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>164</v>
@@ -4226,11 +4226,11 @@
         <v>166</v>
       </c>
       <c r="B45" s="9">
-        <v>46162.625134131944</v>
+        <v>46162.791800798615</v>
       </c>
       <c r="C45" s="10"/>
       <c r="D45" s="9">
-        <v>46198.61601456019</v>
+        <v>46198.78268122685</v>
       </c>
       <c r="E45" s="10" t="s">
         <v>167</v>
@@ -4275,13 +4275,13 @@
         <v>169</v>
       </c>
       <c r="B46" s="5">
-        <v>46162.625454548615</v>
+        <v>46162.79212121527</v>
       </c>
       <c r="C46" s="5">
-        <v>46197.51404692129</v>
+        <v>46197.680713587964</v>
       </c>
       <c r="D46" s="5">
-        <v>46197.51406354167</v>
+        <v>46197.68073020833</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>170</v>
@@ -4340,13 +4340,13 @@
         <v>174</v>
       </c>
       <c r="B47" s="9">
-        <v>46162.625460034724</v>
+        <v>46162.79212670139</v>
       </c>
       <c r="C47" s="9">
-        <v>46198.615996736116</v>
+        <v>46198.78266340277</v>
       </c>
       <c r="D47" s="9">
-        <v>46198.616014907406</v>
+        <v>46198.78268157407</v>
       </c>
       <c r="E47" s="10" t="s">
         <v>175</v>
@@ -4405,13 +4405,13 @@
         <v>178</v>
       </c>
       <c r="B48" s="5">
-        <v>46162.62546642361</v>
+        <v>46162.792133090275</v>
       </c>
       <c r="C48" s="5">
-        <v>46198.61604957176</v>
+        <v>46198.78271623843</v>
       </c>
       <c r="D48" s="5">
-        <v>46198.61606556713</v>
+        <v>46198.7827322338</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>78</v>
@@ -4470,11 +4470,11 @@
         <v>182</v>
       </c>
       <c r="B49" s="9">
-        <v>46162.625480428236</v>
+        <v>46162.79214709491</v>
       </c>
       <c r="C49" s="10"/>
       <c r="D49" s="9">
-        <v>46164.52360884259</v>
+        <v>46164.69027550926</v>
       </c>
       <c r="E49" s="10" t="s">
         <v>183</v>
@@ -4533,11 +4533,11 @@
         <v>187</v>
       </c>
       <c r="B50" s="5">
-        <v>46162.625484108794</v>
+        <v>46162.792150775465</v>
       </c>
       <c r="C50" s="6"/>
       <c r="D50" s="5">
-        <v>46164.523701805556</v>
+        <v>46164.69036847222</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>188</v>
@@ -4586,11 +4586,11 @@
         <v>190</v>
       </c>
       <c r="B51" s="9">
-        <v>46162.62548818287</v>
+        <v>46162.792154849536</v>
       </c>
       <c r="C51" s="10"/>
       <c r="D51" s="9">
-        <v>46164.52369920139</v>
+        <v>46164.69036586805</v>
       </c>
       <c r="E51" s="10" t="s">
         <v>188</v>
@@ -4639,11 +4639,11 @@
         <v>191</v>
       </c>
       <c r="B52" s="5">
-        <v>46162.62549208333</v>
+        <v>46162.79215875</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="5">
-        <v>46164.52369637731</v>
+        <v>46164.69036304398</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>188</v>
@@ -4692,11 +4692,11 @@
         <v>192</v>
       </c>
       <c r="B53" s="9">
-        <v>46162.62549497685</v>
+        <v>46162.79216164352</v>
       </c>
       <c r="C53" s="10"/>
       <c r="D53" s="9">
-        <v>46164.523692268514</v>
+        <v>46164.690358935186</v>
       </c>
       <c r="E53" s="10" t="s">
         <v>188</v>
@@ -4745,11 +4745,11 @@
         <v>193</v>
       </c>
       <c r="B54" s="5">
-        <v>46162.62554516204</v>
+        <v>46162.7922118287</v>
       </c>
       <c r="C54" s="6"/>
       <c r="D54" s="5">
-        <v>46164.500513541665</v>
+        <v>46164.66718020833</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4792,11 +4792,11 @@
         <v>196</v>
       </c>
       <c r="B55" s="9">
-        <v>46162.625553425925</v>
+        <v>46162.7922200926</v>
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="9">
-        <v>46164.52381886574</v>
+        <v>46164.69048553241</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>197</v>
@@ -4855,11 +4855,11 @@
         <v>201</v>
       </c>
       <c r="B56" s="5">
-        <v>46162.62555895833</v>
+        <v>46162.792225625</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46164.52388792824</v>
+        <v>46164.69055459491</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>202</v>
@@ -4918,11 +4918,11 @@
         <v>205</v>
       </c>
       <c r="B57" s="9">
-        <v>46162.625565636576</v>
+        <v>46162.79223230324</v>
       </c>
       <c r="C57" s="10"/>
       <c r="D57" s="9">
-        <v>46164.52381575231</v>
+        <v>46164.690482418984</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>206</v>
@@ -4981,11 +4981,11 @@
         <v>208</v>
       </c>
       <c r="B58" s="5">
-        <v>46162.62557070602</v>
+        <v>46162.79223737269</v>
       </c>
       <c r="C58" s="6"/>
       <c r="D58" s="5">
-        <v>46164.52388519676</v>
+        <v>46164.69055186343</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>209</v>
@@ -5044,11 +5044,11 @@
         <v>211</v>
       </c>
       <c r="B59" s="9">
-        <v>46162.62557578704</v>
+        <v>46162.7922424537</v>
       </c>
       <c r="C59" s="10"/>
       <c r="D59" s="9">
-        <v>46164.52381239583</v>
+        <v>46164.6904790625</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>212</v>
@@ -5107,11 +5107,11 @@
         <v>214</v>
       </c>
       <c r="B60" s="5">
-        <v>46162.62558024305</v>
+        <v>46162.792246909725</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46164.52388266203</v>
+        <v>46164.690549328705</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>213</v>
@@ -5170,11 +5170,11 @@
         <v>215</v>
       </c>
       <c r="B61" s="9">
-        <v>46162.62558502315</v>
+        <v>46162.79225168981</v>
       </c>
       <c r="C61" s="10"/>
       <c r="D61" s="9">
-        <v>46164.50232085648</v>
+        <v>46164.66898752315</v>
       </c>
       <c r="E61" s="10" t="s">
         <v>216</v>
@@ -5217,11 +5217,11 @@
         <v>218</v>
       </c>
       <c r="B62" s="5">
-        <v>46162.6255878125</v>
+        <v>46162.792254479165</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46164.52405841435</v>
+        <v>46164.69072508102</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>219</v>
@@ -5280,11 +5280,11 @@
         <v>222</v>
       </c>
       <c r="B63" s="9">
-        <v>46162.62559255787</v>
+        <v>46162.79225922454</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46164.5240165162</v>
+        <v>46164.69068318287</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>188</v>
@@ -5333,11 +5333,11 @@
         <v>225</v>
       </c>
       <c r="B64" s="5">
-        <v>46162.62559891204</v>
+        <v>46162.792265578704</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46164.52401381945</v>
+        <v>46164.69068048611</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>188</v>
@@ -5386,11 +5386,11 @@
         <v>227</v>
       </c>
       <c r="B65" s="9">
-        <v>46162.62560534722</v>
+        <v>46162.79227201389</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="9">
-        <v>46164.52401086806</v>
+        <v>46164.69067753472</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>188</v>
@@ -5439,11 +5439,11 @@
         <v>230</v>
       </c>
       <c r="B66" s="5">
-        <v>46162.62561162037</v>
+        <v>46162.79227828704</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46164.52400670139</v>
+        <v>46164.69067336805</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>188</v>
@@ -5492,11 +5492,11 @@
         <v>231</v>
       </c>
       <c r="B67" s="9">
-        <v>46162.625655358795</v>
+        <v>46162.79232202546</v>
       </c>
       <c r="C67" s="10"/>
       <c r="D67" s="9">
-        <v>46164.52418478009</v>
+        <v>46164.69085144676</v>
       </c>
       <c r="E67" s="10" t="s">
         <v>232</v>
@@ -5555,11 +5555,11 @@
         <v>233</v>
       </c>
       <c r="B68" s="5">
-        <v>46162.62565987269</v>
+        <v>46162.79232653935</v>
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46198.61605793981</v>
+        <v>46198.782724606484</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>188</v>
@@ -5608,11 +5608,11 @@
         <v>236</v>
       </c>
       <c r="B69" s="9">
-        <v>46162.625665983796</v>
+        <v>46162.79233265047</v>
       </c>
       <c r="C69" s="10"/>
       <c r="D69" s="9">
-        <v>46198.61605696759</v>
+        <v>46198.78272363426</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>188</v>
@@ -5661,11 +5661,11 @@
         <v>237</v>
       </c>
       <c r="B70" s="5">
-        <v>46162.625671539354</v>
+        <v>46162.79233820602</v>
       </c>
       <c r="C70" s="6"/>
       <c r="D70" s="5">
-        <v>46198.61606561343</v>
+        <v>46198.78273228009</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>188</v>
@@ -5714,11 +5714,11 @@
         <v>239</v>
       </c>
       <c r="B71" s="9">
-        <v>46162.62567717592</v>
+        <v>46162.79234384259</v>
       </c>
       <c r="C71" s="10"/>
       <c r="D71" s="9">
-        <v>46198.61606615741</v>
+        <v>46198.782732824075</v>
       </c>
       <c r="E71" s="10" t="s">
         <v>188</v>
@@ -5767,11 +5767,11 @@
         <v>240</v>
       </c>
       <c r="B72" s="5">
-        <v>46162.62574747685</v>
+        <v>46162.79241414352</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46164.52430971064</v>
+        <v>46164.690976377315</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>241</v>
@@ -5830,11 +5830,11 @@
         <v>242</v>
       </c>
       <c r="B73" s="9">
-        <v>46162.62575375</v>
+        <v>46162.79242041666</v>
       </c>
       <c r="C73" s="10"/>
       <c r="D73" s="9">
-        <v>46198.61606674769</v>
+        <v>46198.78273341435</v>
       </c>
       <c r="E73" s="10" t="s">
         <v>188</v>
@@ -5883,11 +5883,11 @@
         <v>244</v>
       </c>
       <c r="B74" s="5">
-        <v>46162.625766550926</v>
+        <v>46162.79243321759</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46198.61605990741</v>
+        <v>46198.78272657408</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>188</v>
@@ -5936,11 +5936,11 @@
         <v>246</v>
       </c>
       <c r="B75" s="9">
-        <v>46162.625772893516</v>
+        <v>46162.79243956019</v>
       </c>
       <c r="C75" s="10"/>
       <c r="D75" s="9">
-        <v>46198.6160604051</v>
+        <v>46198.78272707176</v>
       </c>
       <c r="E75" s="10" t="s">
         <v>188</v>
@@ -5989,11 +5989,11 @@
         <v>248</v>
       </c>
       <c r="B76" s="5">
-        <v>46162.625779849535</v>
+        <v>46162.79244651621</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46198.616055</v>
+        <v>46198.78272166666</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>188</v>
@@ -6042,11 +6042,11 @@
         <v>249</v>
       </c>
       <c r="B77" s="9">
-        <v>46162.625811446764</v>
+        <v>46162.79247811342</v>
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46164.504105960645</v>
+        <v>46164.670772627316</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>194</v>
@@ -6089,11 +6089,11 @@
         <v>251</v>
       </c>
       <c r="B78" s="5">
-        <v>46162.62581513889</v>
+        <v>46162.792481805554</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46171.032529421296</v>
+        <v>46171.19919608797</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>252</v>
@@ -6152,11 +6152,11 @@
         <v>254</v>
       </c>
       <c r="B79" s="9">
-        <v>46162.62582282408</v>
+        <v>46162.79248949074</v>
       </c>
       <c r="C79" s="10"/>
       <c r="D79" s="9">
-        <v>46198.51929491898</v>
+        <v>46198.68596158565</v>
       </c>
       <c r="E79" s="10" t="s">
         <v>255</v>
@@ -6215,11 +6215,11 @@
         <v>257</v>
       </c>
       <c r="B80" s="5">
-        <v>46162.62583023148</v>
+        <v>46162.79249689815</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46198.51902892361</v>
+        <v>46198.68569559028</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>258</v>
@@ -6278,11 +6278,11 @@
         <v>259</v>
       </c>
       <c r="B81" s="9">
-        <v>46162.6258377662</v>
+        <v>46162.79250443287</v>
       </c>
       <c r="C81" s="10"/>
       <c r="D81" s="9">
-        <v>46164.52443952546</v>
+        <v>46164.69110619213</v>
       </c>
       <c r="E81" s="10" t="s">
         <v>260</v>
@@ -6341,11 +6341,11 @@
         <v>262</v>
       </c>
       <c r="B82" s="5">
-        <v>46162.6258428125</v>
+        <v>46162.79250947917</v>
       </c>
       <c r="C82" s="6"/>
       <c r="D82" s="5">
-        <v>46164.517869247684</v>
+        <v>46164.68453591435</v>
       </c>
       <c r="E82" s="6" t="s">
         <v>263</v>
@@ -6388,11 +6388,11 @@
         <v>265</v>
       </c>
       <c r="B83" s="9">
-        <v>46162.62584628472</v>
+        <v>46162.79251295139</v>
       </c>
       <c r="C83" s="10"/>
       <c r="D83" s="9">
-        <v>46164.524581516205</v>
+        <v>46164.69124818287</v>
       </c>
       <c r="E83" s="10" t="s">
         <v>266</v>
@@ -6451,11 +6451,11 @@
         <v>268</v>
       </c>
       <c r="B84" s="5">
-        <v>46162.625862071756</v>
+        <v>46162.79252873843</v>
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46164.52455164352</v>
+        <v>46164.69121831018</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>188</v>
@@ -6504,11 +6504,11 @@
         <v>270</v>
       </c>
       <c r="B85" s="9">
-        <v>46162.62586685186</v>
+        <v>46162.792533518514</v>
       </c>
       <c r="C85" s="10"/>
       <c r="D85" s="9">
-        <v>46164.524549050926</v>
+        <v>46164.6912157176</v>
       </c>
       <c r="E85" s="10" t="s">
         <v>188</v>
@@ -6557,11 +6557,11 @@
         <v>271</v>
       </c>
       <c r="B86" s="5">
-        <v>46162.62587158565</v>
+        <v>46162.79253825231</v>
       </c>
       <c r="C86" s="6"/>
       <c r="D86" s="5">
-        <v>46164.52454670139</v>
+        <v>46164.69121336806</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>188</v>
@@ -6610,11 +6610,11 @@
         <v>273</v>
       </c>
       <c r="B87" s="9">
-        <v>46162.62587653935</v>
+        <v>46162.792543206015</v>
       </c>
       <c r="C87" s="10"/>
       <c r="D87" s="9">
-        <v>46164.524542824074</v>
+        <v>46164.691209490746</v>
       </c>
       <c r="E87" s="10" t="s">
         <v>188</v>
@@ -6663,11 +6663,11 @@
         <v>275</v>
       </c>
       <c r="B88" s="5">
-        <v>46162.62594607639</v>
+        <v>46162.792612743055</v>
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46164.524713032406</v>
+        <v>46164.69137969907</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>276</v>
@@ -6726,11 +6726,11 @@
         <v>277</v>
       </c>
       <c r="B89" s="9">
-        <v>46162.62595178241</v>
+        <v>46162.79261844908</v>
       </c>
       <c r="C89" s="10"/>
       <c r="D89" s="9">
-        <v>46198.616074606485</v>
+        <v>46198.78274127315</v>
       </c>
       <c r="E89" s="10" t="s">
         <v>188</v>
@@ -6779,11 +6779,11 @@
         <v>280</v>
       </c>
       <c r="B90" s="5">
-        <v>46162.62595806713</v>
+        <v>46162.7926247338</v>
       </c>
       <c r="C90" s="6"/>
       <c r="D90" s="5">
-        <v>46198.61605556713</v>
+        <v>46198.782722233795</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>188</v>
@@ -6832,11 +6832,11 @@
         <v>281</v>
       </c>
       <c r="B91" s="9">
-        <v>46162.6259640162</v>
+        <v>46162.792630682874</v>
       </c>
       <c r="C91" s="10"/>
       <c r="D91" s="9">
-        <v>46198.61605844907</v>
+        <v>46198.78272511574</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>188</v>
@@ -6885,11 +6885,11 @@
         <v>283</v>
       </c>
       <c r="B92" s="5">
-        <v>46162.62597111111</v>
+        <v>46162.79263777778</v>
       </c>
       <c r="C92" s="6"/>
       <c r="D92" s="5">
-        <v>46198.61605744213</v>
+        <v>46198.782724108794</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>188</v>
@@ -6938,11 +6938,11 @@
         <v>284</v>
       </c>
       <c r="B93" s="9">
-        <v>46162.626019375</v>
+        <v>46162.79268604166</v>
       </c>
       <c r="C93" s="10"/>
       <c r="D93" s="9">
-        <v>46164.524833738426</v>
+        <v>46164.6915004051</v>
       </c>
       <c r="E93" s="10" t="s">
         <v>285</v>
@@ -7001,11 +7001,11 @@
         <v>286</v>
       </c>
       <c r="B94" s="5">
-        <v>46162.62602403935</v>
+        <v>46162.79269070602</v>
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46198.616056053244</v>
+        <v>46198.78272271991</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>188</v>
@@ -7054,11 +7054,11 @@
         <v>288</v>
       </c>
       <c r="B95" s="9">
-        <v>46162.626030405096</v>
+        <v>46162.79269707176</v>
       </c>
       <c r="C95" s="10"/>
       <c r="D95" s="9">
-        <v>46198.616058935186</v>
+        <v>46198.78272560185</v>
       </c>
       <c r="E95" s="10" t="s">
         <v>188</v>
@@ -7107,11 +7107,11 @@
         <v>290</v>
       </c>
       <c r="B96" s="5">
-        <v>46162.62603690972</v>
+        <v>46162.792703576386</v>
       </c>
       <c r="C96" s="6"/>
       <c r="D96" s="5">
-        <v>46198.61606707176</v>
+        <v>46198.78273373842</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>188</v>
@@ -7160,11 +7160,11 @@
         <v>292</v>
       </c>
       <c r="B97" s="9">
-        <v>46162.62604379629</v>
+        <v>46162.79271046296</v>
       </c>
       <c r="C97" s="10"/>
       <c r="D97" s="9">
-        <v>46198.61605939815</v>
+        <v>46198.78272606482</v>
       </c>
       <c r="E97" s="10" t="s">
         <v>188</v>
@@ -7213,11 +7213,11 @@
         <v>295</v>
       </c>
       <c r="B98" s="5">
-        <v>46162.626078194444</v>
+        <v>46162.792744861115</v>
       </c>
       <c r="C98" s="6"/>
       <c r="D98" s="5">
-        <v>46164.52495327547</v>
+        <v>46164.691619942125</v>
       </c>
       <c r="E98" s="6" t="s">
         <v>296</v>
@@ -7276,11 +7276,11 @@
         <v>297</v>
       </c>
       <c r="B99" s="9">
-        <v>46162.62608315972</v>
+        <v>46162.79274982639</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="9">
-        <v>46198.616060879634</v>
+        <v>46198.78272754629</v>
       </c>
       <c r="E99" s="10" t="s">
         <v>188</v>
@@ -7329,11 +7329,11 @@
         <v>300</v>
       </c>
       <c r="B100" s="5">
-        <v>46162.626088923615</v>
+        <v>46162.79275559028</v>
       </c>
       <c r="C100" s="6"/>
       <c r="D100" s="5">
-        <v>46198.61605643519</v>
+        <v>46198.78272310185</v>
       </c>
       <c r="E100" s="6" t="s">
         <v>188</v>
@@ -7382,11 +7382,11 @@
         <v>301</v>
       </c>
       <c r="B101" s="9">
-        <v>46162.62609451389</v>
+        <v>46162.79276118056</v>
       </c>
       <c r="C101" s="10"/>
       <c r="D101" s="9">
-        <v>46198.61606122685</v>
+        <v>46198.782727893515</v>
       </c>
       <c r="E101" s="10" t="s">
         <v>188</v>
@@ -7435,11 +7435,11 @@
         <v>303</v>
       </c>
       <c r="B102" s="5">
-        <v>46162.62610108797</v>
+        <v>46162.792767754625</v>
       </c>
       <c r="C102" s="6"/>
       <c r="D102" s="5">
-        <v>46198.61606172453</v>
+        <v>46198.782728391205</v>
       </c>
       <c r="E102" s="6" t="s">
         <v>188</v>
@@ -7488,11 +7488,11 @@
         <v>305</v>
       </c>
       <c r="B103" s="9">
-        <v>46162.62619030093</v>
+        <v>46162.79285696759</v>
       </c>
       <c r="C103" s="10"/>
       <c r="D103" s="9">
-        <v>46164.525072881945</v>
+        <v>46164.69173954861</v>
       </c>
       <c r="E103" s="10" t="s">
         <v>306</v>
@@ -7551,11 +7551,11 @@
         <v>307</v>
       </c>
       <c r="B104" s="5">
-        <v>46162.6261958449</v>
+        <v>46162.792862511575</v>
       </c>
       <c r="C104" s="6"/>
       <c r="D104" s="5">
-        <v>46164.525042002315</v>
+        <v>46164.69170866898</v>
       </c>
       <c r="E104" s="6" t="s">
         <v>188</v>
@@ -7604,11 +7604,11 @@
         <v>309</v>
       </c>
       <c r="B105" s="9">
-        <v>46162.62620145833</v>
+        <v>46162.792868125005</v>
       </c>
       <c r="C105" s="10"/>
       <c r="D105" s="9">
-        <v>46164.52503929398</v>
+        <v>46164.69170596065</v>
       </c>
       <c r="E105" s="10" t="s">
         <v>188</v>
@@ -7657,11 +7657,11 @@
         <v>311</v>
       </c>
       <c r="B106" s="5">
-        <v>46162.62620708333</v>
+        <v>46162.792873750004</v>
       </c>
       <c r="C106" s="6"/>
       <c r="D106" s="5">
-        <v>46164.525036273146</v>
+        <v>46164.69170293982</v>
       </c>
       <c r="E106" s="6" t="s">
         <v>188</v>
@@ -7710,11 +7710,11 @@
         <v>312</v>
       </c>
       <c r="B107" s="9">
-        <v>46162.62621266204</v>
+        <v>46162.7928793287</v>
       </c>
       <c r="C107" s="10"/>
       <c r="D107" s="9">
-        <v>46164.52503152778</v>
+        <v>46164.691698194445</v>
       </c>
       <c r="E107" s="10" t="s">
         <v>188</v>
@@ -7763,11 +7763,11 @@
         <v>313</v>
       </c>
       <c r="B108" s="5">
-        <v>46162.62624103009</v>
+        <v>46162.792907696756</v>
       </c>
       <c r="C108" s="6"/>
       <c r="D108" s="5">
-        <v>46164.52519069445</v>
+        <v>46164.69185736111</v>
       </c>
       <c r="E108" s="6" t="s">
         <v>314</v>
@@ -7824,11 +7824,11 @@
         <v>316</v>
       </c>
       <c r="B109" s="9">
-        <v>46162.62624622685</v>
+        <v>46162.79291289352</v>
       </c>
       <c r="C109" s="10"/>
       <c r="D109" s="9">
-        <v>46164.52515765047</v>
+        <v>46164.69182431713</v>
       </c>
       <c r="E109" s="10" t="s">
         <v>188</v>
@@ -7877,11 +7877,11 @@
         <v>318</v>
       </c>
       <c r="B110" s="5">
-        <v>46162.626250914356</v>
+        <v>46162.79291758101</v>
       </c>
       <c r="C110" s="6"/>
       <c r="D110" s="5">
-        <v>46164.52515489583</v>
+        <v>46164.691821562505</v>
       </c>
       <c r="E110" s="6" t="s">
         <v>188</v>
@@ -7930,11 +7930,11 @@
         <v>319</v>
       </c>
       <c r="B111" s="9">
-        <v>46162.626255787036</v>
+        <v>46162.79292245371</v>
       </c>
       <c r="C111" s="10"/>
       <c r="D111" s="9">
-        <v>46164.52515248842</v>
+        <v>46164.691819155094</v>
       </c>
       <c r="E111" s="10" t="s">
         <v>188</v>
@@ -7983,11 +7983,11 @@
         <v>320</v>
       </c>
       <c r="B112" s="5">
-        <v>46162.62626590278</v>
+        <v>46162.79293256944</v>
       </c>
       <c r="C112" s="6"/>
       <c r="D112" s="5">
-        <v>46164.52514842592</v>
+        <v>46164.69181509259</v>
       </c>
       <c r="E112" s="6" t="s">
         <v>188</v>
@@ -8036,11 +8036,11 @@
         <v>321</v>
       </c>
       <c r="B113" s="9">
-        <v>46162.626337395835</v>
+        <v>46162.7930040625</v>
       </c>
       <c r="C113" s="10"/>
       <c r="D113" s="9">
-        <v>46164.518794965275</v>
+        <v>46164.68546163195</v>
       </c>
       <c r="E113" s="10" t="s">
         <v>322</v>
@@ -8083,11 +8083,11 @@
         <v>324</v>
       </c>
       <c r="B114" s="5">
-        <v>46162.626341400464</v>
+        <v>46162.79300806713</v>
       </c>
       <c r="C114" s="6"/>
       <c r="D114" s="5">
-        <v>46164.525584849536</v>
+        <v>46164.6922515162</v>
       </c>
       <c r="E114" s="6" t="s">
         <v>325</v>
@@ -8146,11 +8146,11 @@
         <v>329</v>
       </c>
       <c r="B115" s="9">
-        <v>46162.62635180556</v>
+        <v>46162.79301847222</v>
       </c>
       <c r="C115" s="10"/>
       <c r="D115" s="9">
-        <v>46164.525564814816</v>
+        <v>46164.69223148148</v>
       </c>
       <c r="E115" s="10" t="s">
         <v>188</v>
@@ -8199,11 +8199,11 @@
         <v>331</v>
       </c>
       <c r="B116" s="5">
-        <v>46162.626358587964</v>
+        <v>46162.79302525463</v>
       </c>
       <c r="C116" s="6"/>
       <c r="D116" s="5">
-        <v>46164.52556148148</v>
+        <v>46164.69222814815</v>
       </c>
       <c r="E116" s="6" t="s">
         <v>188</v>
@@ -8252,11 +8252,11 @@
         <v>332</v>
       </c>
       <c r="B117" s="9">
-        <v>46162.6263634375</v>
+        <v>46162.79303010416</v>
       </c>
       <c r="C117" s="10"/>
       <c r="D117" s="9">
-        <v>46164.525558587964</v>
+        <v>46164.69222525463</v>
       </c>
       <c r="E117" s="10" t="s">
         <v>188</v>
@@ -8305,11 +8305,11 @@
         <v>334</v>
       </c>
       <c r="B118" s="5">
-        <v>46162.62636815972</v>
+        <v>46162.79303482639</v>
       </c>
       <c r="C118" s="6"/>
       <c r="D118" s="5">
-        <v>46164.52555344907</v>
+        <v>46164.69222011574</v>
       </c>
       <c r="E118" s="6" t="s">
         <v>188</v>
@@ -8358,11 +8358,11 @@
         <v>335</v>
       </c>
       <c r="B119" s="9">
-        <v>46162.6263962963</v>
+        <v>46162.79306296296</v>
       </c>
       <c r="C119" s="10"/>
       <c r="D119" s="9">
-        <v>46164.52570229166</v>
+        <v>46164.692368958335</v>
       </c>
       <c r="E119" s="10" t="s">
         <v>336</v>
@@ -8421,11 +8421,11 @@
         <v>337</v>
       </c>
       <c r="B120" s="5">
-        <v>46162.62640114583</v>
+        <v>46162.7930678125</v>
       </c>
       <c r="C120" s="6"/>
       <c r="D120" s="5">
-        <v>46164.52566752315</v>
+        <v>46164.692334189815</v>
       </c>
       <c r="E120" s="6" t="s">
         <v>188</v>
@@ -8474,11 +8474,11 @@
         <v>339</v>
       </c>
       <c r="B121" s="9">
-        <v>46162.626405613424</v>
+        <v>46162.793072280096</v>
       </c>
       <c r="C121" s="10"/>
       <c r="D121" s="9">
-        <v>46164.52566484954</v>
+        <v>46164.6923315162</v>
       </c>
       <c r="E121" s="10" t="s">
         <v>188</v>
@@ -8527,11 +8527,11 @@
         <v>340</v>
       </c>
       <c r="B122" s="5">
-        <v>46162.62641030093</v>
+        <v>46162.79307696759</v>
       </c>
       <c r="C122" s="6"/>
       <c r="D122" s="5">
-        <v>46164.525662141205</v>
+        <v>46164.69232880787</v>
       </c>
       <c r="E122" s="6" t="s">
         <v>188</v>
@@ -8580,11 +8580,11 @@
         <v>342</v>
       </c>
       <c r="B123" s="9">
-        <v>46162.62641509259</v>
+        <v>46162.79308175926</v>
       </c>
       <c r="C123" s="10"/>
       <c r="D123" s="9">
-        <v>46164.52565760417</v>
+        <v>46164.69232427083</v>
       </c>
       <c r="E123" s="10" t="s">
         <v>188</v>
@@ -8633,11 +8633,11 @@
         <v>343</v>
       </c>
       <c r="B124" s="5">
-        <v>46162.626479583334</v>
+        <v>46162.79314625</v>
       </c>
       <c r="C124" s="6"/>
       <c r="D124" s="5">
-        <v>46164.52582030093</v>
+        <v>46164.69248696759</v>
       </c>
       <c r="E124" s="6" t="s">
         <v>344</v>
@@ -8696,11 +8696,11 @@
         <v>345</v>
       </c>
       <c r="B125" s="9">
-        <v>46162.626484884255</v>
+        <v>46162.793151550926</v>
       </c>
       <c r="C125" s="10"/>
       <c r="D125" s="9">
-        <v>46164.525794085646</v>
+        <v>46164.69246075231</v>
       </c>
       <c r="E125" s="10" t="s">
         <v>188</v>
@@ -8749,11 +8749,11 @@
         <v>347</v>
       </c>
       <c r="B126" s="5">
-        <v>46162.6264921875</v>
+        <v>46162.79315885417</v>
       </c>
       <c r="C126" s="6"/>
       <c r="D126" s="5">
-        <v>46164.52579143518</v>
+        <v>46164.692458101854</v>
       </c>
       <c r="E126" s="6" t="s">
         <v>188</v>
@@ -8802,11 +8802,11 @@
         <v>348</v>
       </c>
       <c r="B127" s="9">
-        <v>46162.62649834491</v>
+        <v>46162.79316501158</v>
       </c>
       <c r="C127" s="10"/>
       <c r="D127" s="9">
-        <v>46164.52578892361</v>
+        <v>46164.69245559028</v>
       </c>
       <c r="E127" s="10" t="s">
         <v>188</v>
@@ -8855,11 +8855,11 @@
         <v>350</v>
       </c>
       <c r="B128" s="5">
-        <v>46162.62650319445</v>
+        <v>46162.79316986111</v>
       </c>
       <c r="C128" s="6"/>
       <c r="D128" s="5">
-        <v>46164.525784618054</v>
+        <v>46164.69245128472</v>
       </c>
       <c r="E128" s="6" t="s">
         <v>188</v>
@@ -8908,11 +8908,11 @@
         <v>352</v>
       </c>
       <c r="B129" s="9">
-        <v>46162.62653059028</v>
+        <v>46162.79319725695</v>
       </c>
       <c r="C129" s="10"/>
       <c r="D129" s="9">
-        <v>46164.52595978009</v>
+        <v>46164.69262644676</v>
       </c>
       <c r="E129" s="10" t="s">
         <v>353</v>
@@ -8971,11 +8971,11 @@
         <v>355</v>
       </c>
       <c r="B130" s="5">
-        <v>46162.62653543982</v>
+        <v>46162.79320210648</v>
       </c>
       <c r="C130" s="6"/>
       <c r="D130" s="5">
-        <v>46164.52592063657</v>
+        <v>46164.692587303245</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>188</v>
@@ -9024,11 +9024,11 @@
         <v>356</v>
       </c>
       <c r="B131" s="9">
-        <v>46162.62653944445</v>
+        <v>46162.793206111106</v>
       </c>
       <c r="C131" s="10"/>
       <c r="D131" s="9">
-        <v>46164.52591784722</v>
+        <v>46164.69258451389</v>
       </c>
       <c r="E131" s="10" t="s">
         <v>188</v>
@@ -9077,11 +9077,11 @@
         <v>357</v>
       </c>
       <c r="B132" s="5">
-        <v>46162.62654328704</v>
+        <v>46162.7932099537</v>
       </c>
       <c r="C132" s="6"/>
       <c r="D132" s="5">
-        <v>46164.52591521991</v>
+        <v>46164.69258188657</v>
       </c>
       <c r="E132" s="6" t="s">
         <v>188</v>
@@ -9130,11 +9130,11 @@
         <v>358</v>
       </c>
       <c r="B133" s="9">
-        <v>46162.62654733796</v>
+        <v>46162.79321400463</v>
       </c>
       <c r="C133" s="10"/>
       <c r="D133" s="9">
-        <v>46164.525910752316</v>
+        <v>46164.69257741898</v>
       </c>
       <c r="E133" s="10" t="s">
         <v>188</v>
@@ -9183,11 +9183,11 @@
         <v>359</v>
       </c>
       <c r="B134" s="5">
-        <v>46162.62657099537</v>
+        <v>46162.79323766204</v>
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46164.51925614583</v>
+        <v>46164.685922812496</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>360</v>
@@ -9230,11 +9230,11 @@
         <v>362</v>
       </c>
       <c r="B135" s="9">
-        <v>46162.62657396991</v>
+        <v>46162.79324063657</v>
       </c>
       <c r="C135" s="10"/>
       <c r="D135" s="9">
-        <v>46164.526027175925</v>
+        <v>46164.69269384259</v>
       </c>
       <c r="E135" s="10" t="s">
         <v>363</v>
@@ -9293,11 +9293,11 @@
         <v>366</v>
       </c>
       <c r="B136" s="5">
-        <v>46162.62657862269</v>
+        <v>46162.79324528935</v>
       </c>
       <c r="C136" s="6"/>
       <c r="D136" s="5">
-        <v>46197.61014160879</v>
+        <v>46197.77680827546</v>
       </c>
       <c r="E136" s="6" t="s">
         <v>367</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-14 14:54 UTC
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1599" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1600" uniqueCount="367">
   <si>
     <t xml:space="preserve"> 50001553- ZITRON COLOMBIA ARIS MINING SEGOVIA - OT4326</t>
   </si>
@@ -685,9 +685,6 @@
     <t xml:space="preserve">Control de calidad corte laser </t>
   </si>
   <si>
-    <t>Recepcion materiales corte laser,Recepcion Materiales corte plasma</t>
-  </si>
-  <si>
     <t>Bodega:,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4</t>
   </si>
   <si>
@@ -697,13 +694,10 @@
     <t>Recepcion Materiales corte plasma</t>
   </si>
   <si>
-    <t>Control de calidad corte laser ,Control de calidad Corte plasma</t>
+    <t>Control de calidad Corte plasma</t>
   </si>
   <si>
     <t>1214982595357416</t>
-  </si>
-  <si>
-    <t>Control de calidad Corte plasma</t>
   </si>
   <si>
     <t>OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4,OT 4326- ZVN 1-12-55/4</t>
@@ -4830,9 +4824,11 @@
       <c r="B54" s="5">
         <v>46162.7922118287</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46217.58831976852</v>
+      </c>
       <c r="D54" s="5">
-        <v>46164.66718020833</v>
+        <v>46217.58833277778</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>195</v>
@@ -4867,8 +4863,12 @@
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
       <c r="S54" s="6"/>
-      <c r="T54" s="6"/>
-      <c r="U54" s="6"/>
+      <c r="T54" s="6">
+        <v>1</v>
+      </c>
+      <c r="U54" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
@@ -4877,9 +4877,11 @@
       <c r="B55" s="9">
         <v>46162.7922200926</v>
       </c>
-      <c r="C55" s="10"/>
+      <c r="C55" s="9">
+        <v>46217.587680173616</v>
+      </c>
       <c r="D55" s="9">
-        <v>46209.81742680556</v>
+        <v>46217.58769918981</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>198</v>
@@ -4927,10 +4929,10 @@
         <v>53</v>
       </c>
       <c r="T55" s="10">
-        <v>0</v>
-      </c>
-      <c r="U55" s="12" t="s">
-        <v>46</v>
+        <v>1</v>
+      </c>
+      <c r="U55" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
@@ -4940,9 +4942,11 @@
       <c r="B56" s="5">
         <v>46162.792225625</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46217.58784472222</v>
+      </c>
       <c r="D56" s="5">
-        <v>46164.69055459491</v>
+        <v>46217.58785994213</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>203</v>
@@ -4975,10 +4979,10 @@
         <v>195</v>
       </c>
       <c r="O56" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="P56" s="6" t="s">
         <v>204</v>
-      </c>
-      <c r="P56" s="6" t="s">
-        <v>205</v>
       </c>
       <c r="Q56" s="5">
         <v>46254</v>
@@ -4990,25 +4994,27 @@
         <v>53</v>
       </c>
       <c r="T56" s="6">
-        <v>0</v>
-      </c>
-      <c r="U56" s="11" t="s">
-        <v>101</v>
+        <v>1</v>
+      </c>
+      <c r="U56" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B57" s="9">
         <v>46162.79223230324</v>
       </c>
-      <c r="C57" s="10"/>
+      <c r="C57" s="9">
+        <v>46217.58814275463</v>
+      </c>
       <c r="D57" s="9">
-        <v>46209.81754253472</v>
+        <v>46217.58816130787</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
@@ -5041,7 +5047,7 @@
         <v>143</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q57" s="9">
         <v>46252</v>
@@ -5053,25 +5059,27 @@
         <v>53</v>
       </c>
       <c r="T57" s="10">
-        <v>0</v>
-      </c>
-      <c r="U57" s="12" t="s">
-        <v>46</v>
+        <v>1</v>
+      </c>
+      <c r="U57" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B58" s="5">
         <v>46162.79223737269</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46217.58818075231</v>
+      </c>
       <c r="D58" s="5">
-        <v>46164.69055186343</v>
+        <v>46217.588195752316</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>26</v>
@@ -5101,10 +5109,10 @@
         <v>195</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="P58" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="Q58" s="5">
         <v>46254</v>
@@ -5116,25 +5124,27 @@
         <v>53</v>
       </c>
       <c r="T58" s="6">
-        <v>0</v>
-      </c>
-      <c r="U58" s="11" t="s">
-        <v>101</v>
+        <v>1</v>
+      </c>
+      <c r="U58" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B59" s="9">
         <v>46162.7922424537</v>
       </c>
-      <c r="C59" s="10"/>
+      <c r="C59" s="9">
+        <v>46217.588267430554</v>
+      </c>
       <c r="D59" s="9">
-        <v>46205.61214489583</v>
+        <v>46217.58828952546</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>26</v>
@@ -5167,7 +5177,7 @@
         <v>165</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="Q59" s="9">
         <v>46252</v>
@@ -5179,25 +5189,27 @@
         <v>53</v>
       </c>
       <c r="T59" s="10">
-        <v>0</v>
-      </c>
-      <c r="U59" s="12" t="s">
-        <v>46</v>
+        <v>1</v>
+      </c>
+      <c r="U59" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B60" s="5">
         <v>46162.792246909725</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46217.58830322917</v>
+      </c>
       <c r="D60" s="5">
-        <v>46164.690549328705</v>
+        <v>46217.58832047453</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="F60" s="6" t="s">
         <v>26</v>
@@ -5227,10 +5239,10 @@
         <v>195</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="Q60" s="5">
         <v>46254</v>
@@ -5242,15 +5254,15 @@
         <v>53</v>
       </c>
       <c r="T60" s="6">
-        <v>0</v>
-      </c>
-      <c r="U60" s="11" t="s">
-        <v>101</v>
+        <v>1</v>
+      </c>
+      <c r="U60" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B61" s="9">
         <v>46162.79225168981</v>
@@ -5260,7 +5272,7 @@
         <v>46164.66898752315</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>25</v>
@@ -5284,7 +5296,7 @@
         <v>26</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="P61" s="10" t="s">
         <v>26</v>
@@ -5297,7 +5309,7 @@
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B62" s="5">
         <v>46162.792254479165</v>
@@ -5307,16 +5319,16 @@
         <v>46164.69072508102</v>
       </c>
       <c r="E62" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G62" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>220</v>
-      </c>
-      <c r="F62" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G62" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>222</v>
       </c>
       <c r="I62" s="5">
         <v>46258</v>
@@ -5334,13 +5346,13 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P62" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="Q62" s="5">
         <v>46258</v>
@@ -5360,14 +5372,14 @@
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B63" s="9">
         <v>46162.79225922454</v>
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46164.69068318287</v>
+        <v>46217.58831070602</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>189</v>
@@ -5376,10 +5388,10 @@
         <v>26</v>
       </c>
       <c r="G63" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I63" s="9">
         <v>46258</v>
@@ -5397,13 +5409,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="Q63" s="10"/>
       <c r="R63" s="10"/>
@@ -5413,14 +5425,14 @@
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B64" s="5">
         <v>46162.792265578704</v>
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46164.69068048611</v>
+        <v>46217.588311886575</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>189</v>
@@ -5429,10 +5441,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I64" s="5">
         <v>46258</v>
@@ -5450,13 +5462,13 @@
         <v>26</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="P64" s="6" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="Q64" s="6"/>
       <c r="R64" s="6"/>
@@ -5466,14 +5478,14 @@
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B65" s="9">
         <v>46162.79227201389</v>
       </c>
       <c r="C65" s="10"/>
       <c r="D65" s="9">
-        <v>46164.69067753472</v>
+        <v>46217.58831295139</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>189</v>
@@ -5482,10 +5494,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I65" s="9">
         <v>46258</v>
@@ -5503,13 +5515,13 @@
         <v>26</v>
       </c>
       <c r="N65" s="10" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="O65" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="P65" s="10" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="Q65" s="10"/>
       <c r="R65" s="10"/>
@@ -5519,14 +5531,14 @@
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B66" s="5">
         <v>46162.79227828704</v>
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46164.69067336805</v>
+        <v>46217.58831400463</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>189</v>
@@ -5535,10 +5547,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I66" s="5">
         <v>46258</v>
@@ -5556,13 +5568,13 @@
         <v>26</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="P66" s="6" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="Q66" s="6"/>
       <c r="R66" s="6"/>
@@ -5572,7 +5584,7 @@
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B67" s="9">
         <v>46162.79232202546</v>
@@ -5582,16 +5594,16 @@
         <v>46164.69085144676</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G67" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I67" s="9">
         <v>46267</v>
@@ -5609,13 +5621,13 @@
         <v>26</v>
       </c>
       <c r="N67" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="O67" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P67" s="10" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="Q67" s="9">
         <v>46267</v>
@@ -5635,7 +5647,7 @@
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B68" s="5">
         <v>46162.79232653935</v>
@@ -5651,10 +5663,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I68" s="5">
         <v>46267</v>
@@ -5672,13 +5684,13 @@
         <v>26</v>
       </c>
       <c r="N68" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="O68" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="O68" s="6" t="s">
-        <v>235</v>
-      </c>
       <c r="P68" s="6" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="Q68" s="6"/>
       <c r="R68" s="6"/>
@@ -5688,7 +5700,7 @@
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="8" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B69" s="9">
         <v>46162.79233265047</v>
@@ -5704,10 +5716,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I69" s="9">
         <v>46267</v>
@@ -5725,13 +5737,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="O69" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="O69" s="10" t="s">
-        <v>235</v>
-      </c>
       <c r="P69" s="10" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="Q69" s="10"/>
       <c r="R69" s="10"/>
@@ -5741,7 +5753,7 @@
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B70" s="5">
         <v>46162.79233820602</v>
@@ -5757,10 +5769,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I70" s="5">
         <v>46267</v>
@@ -5778,13 +5790,13 @@
         <v>26</v>
       </c>
       <c r="N70" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="O70" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="O70" s="6" t="s">
-        <v>235</v>
-      </c>
       <c r="P70" s="6" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="Q70" s="6"/>
       <c r="R70" s="6"/>
@@ -5794,7 +5806,7 @@
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="8" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B71" s="9">
         <v>46162.79234384259</v>
@@ -5810,10 +5822,10 @@
         <v>26</v>
       </c>
       <c r="G71" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H71" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I71" s="9">
         <v>46267</v>
@@ -5831,13 +5843,13 @@
         <v>26</v>
       </c>
       <c r="N71" s="10" t="s">
+        <v>231</v>
+      </c>
+      <c r="O71" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="O71" s="10" t="s">
-        <v>235</v>
-      </c>
       <c r="P71" s="10" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="Q71" s="10"/>
       <c r="R71" s="10"/>
@@ -5847,7 +5859,7 @@
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B72" s="5">
         <v>46162.79241414352</v>
@@ -5857,7 +5869,7 @@
         <v>46164.690976377315</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
@@ -5884,13 +5896,13 @@
         <v>26</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P72" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="Q72" s="5">
         <v>46289</v>
@@ -5910,7 +5922,7 @@
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="8" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B73" s="9">
         <v>46162.79242041666</v>
@@ -5947,13 +5959,13 @@
         <v>26</v>
       </c>
       <c r="N73" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="O73" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="P73" s="10" t="s">
         <v>242</v>
-      </c>
-      <c r="O73" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="P73" s="10" t="s">
-        <v>244</v>
       </c>
       <c r="Q73" s="10"/>
       <c r="R73" s="10"/>
@@ -5963,7 +5975,7 @@
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B74" s="5">
         <v>46162.79243321759</v>
@@ -6000,13 +6012,13 @@
         <v>26</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="Q74" s="6"/>
       <c r="R74" s="6"/>
@@ -6016,7 +6028,7 @@
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="8" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B75" s="9">
         <v>46162.79243956019</v>
@@ -6053,13 +6065,13 @@
         <v>26</v>
       </c>
       <c r="N75" s="10" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="O75" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="P75" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="Q75" s="10"/>
       <c r="R75" s="10"/>
@@ -6069,7 +6081,7 @@
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B76" s="5">
         <v>46162.79244651621</v>
@@ -6106,13 +6118,13 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="P76" s="6" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="Q76" s="6"/>
       <c r="R76" s="6"/>
@@ -6122,7 +6134,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="8" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B77" s="9">
         <v>46162.79247811342</v>
@@ -6156,7 +6168,7 @@
         <v>26</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>26</v>
@@ -6171,7 +6183,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B78" s="5">
         <v>46162.792481805554</v>
@@ -6183,7 +6195,7 @@
         <v>46212.65536587963</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
@@ -6216,7 +6228,7 @@
         <v>112</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="Q78" s="5">
         <v>46169</v>
@@ -6236,7 +6248,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B79" s="9">
         <v>46162.79248949074</v>
@@ -6248,7 +6260,7 @@
         <v>46212.655404537036</v>
       </c>
       <c r="E79" s="10" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>26</v>
@@ -6281,7 +6293,7 @@
         <v>103</v>
       </c>
       <c r="P79" s="10" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="Q79" s="9">
         <v>46279</v>
@@ -6301,7 +6313,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B80" s="5">
         <v>46162.79249689815</v>
@@ -6313,7 +6325,7 @@
         <v>46212.65570653936</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
@@ -6346,7 +6358,7 @@
         <v>121</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="Q80" s="5">
         <v>46302</v>
@@ -6366,7 +6378,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B81" s="9">
         <v>46162.79250443287</v>
@@ -6376,7 +6388,7 @@
         <v>46209.62459446759</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
@@ -6409,7 +6421,7 @@
         <v>153</v>
       </c>
       <c r="P81" s="10" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="Q81" s="9">
         <v>46280</v>
@@ -6429,7 +6441,7 @@
     </row>
     <row r="82" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B82" s="5">
         <v>46162.79250947917</v>
@@ -6439,7 +6451,7 @@
         <v>46164.68453591435</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>25</v>
@@ -6463,7 +6475,7 @@
         <v>26</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>26</v>
@@ -6476,7 +6488,7 @@
     </row>
     <row r="83" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B83" s="9">
         <v>46162.79251295139</v>
@@ -6486,7 +6498,7 @@
         <v>46164.69124818287</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
@@ -6513,13 +6525,13 @@
         <v>26</v>
       </c>
       <c r="N83" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="P83" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="Q83" s="9">
         <v>46293</v>
@@ -6539,7 +6551,7 @@
     </row>
     <row r="84" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B84" s="5">
         <v>46162.79252873843</v>
@@ -6576,10 +6588,10 @@
         <v>26</v>
       </c>
       <c r="N84" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>26</v>
@@ -6592,7 +6604,7 @@
     </row>
     <row r="85" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="B85" s="9">
         <v>46162.792533518514</v>
@@ -6629,10 +6641,10 @@
         <v>26</v>
       </c>
       <c r="N85" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="P85" s="10" t="s">
         <v>26</v>
@@ -6645,7 +6657,7 @@
     </row>
     <row r="86" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B86" s="5">
         <v>46162.79253825231</v>
@@ -6682,13 +6694,13 @@
         <v>26</v>
       </c>
       <c r="N86" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="O86" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P86" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="Q86" s="6"/>
       <c r="R86" s="6"/>
@@ -6698,7 +6710,7 @@
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="8" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B87" s="9">
         <v>46162.792543206015</v>
@@ -6735,13 +6747,13 @@
         <v>26</v>
       </c>
       <c r="N87" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="O87" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P87" s="10" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="Q87" s="10"/>
       <c r="R87" s="10"/>
@@ -6751,7 +6763,7 @@
     </row>
     <row r="88" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="4" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B88" s="5">
         <v>46162.792612743055</v>
@@ -6761,7 +6773,7 @@
         <v>46164.69137969907</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
@@ -6788,13 +6800,13 @@
         <v>26</v>
       </c>
       <c r="N88" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O88" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P88" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="Q88" s="5">
         <v>46311</v>
@@ -6814,7 +6826,7 @@
     </row>
     <row r="89" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="8" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B89" s="9">
         <v>46162.79261844908</v>
@@ -6851,13 +6863,13 @@
         <v>26</v>
       </c>
       <c r="N89" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="O89" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="O89" s="10" t="s">
-        <v>279</v>
-      </c>
       <c r="P89" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="Q89" s="10"/>
       <c r="R89" s="10"/>
@@ -6867,7 +6879,7 @@
     </row>
     <row r="90" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="4" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B90" s="5">
         <v>46162.7926247338</v>
@@ -6904,13 +6916,13 @@
         <v>26</v>
       </c>
       <c r="N90" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="O90" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="O90" s="6" t="s">
-        <v>279</v>
-      </c>
       <c r="P90" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="Q90" s="6"/>
       <c r="R90" s="6"/>
@@ -6920,7 +6932,7 @@
     </row>
     <row r="91" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="8" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B91" s="9">
         <v>46162.792630682874</v>
@@ -6957,13 +6969,13 @@
         <v>26</v>
       </c>
       <c r="N91" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="O91" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="P91" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="Q91" s="10"/>
       <c r="R91" s="10"/>
@@ -6973,7 +6985,7 @@
     </row>
     <row r="92" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="4" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="B92" s="5">
         <v>46162.79263777778</v>
@@ -7010,13 +7022,13 @@
         <v>26</v>
       </c>
       <c r="N92" s="6" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="P92" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="Q92" s="6"/>
       <c r="R92" s="6"/>
@@ -7026,7 +7038,7 @@
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="8" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="B93" s="9">
         <v>46162.79268604166</v>
@@ -7036,7 +7048,7 @@
         <v>46164.6915004051</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
@@ -7063,13 +7075,13 @@
         <v>26</v>
       </c>
       <c r="N93" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O93" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P93" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="Q93" s="9">
         <v>46315</v>
@@ -7089,7 +7101,7 @@
     </row>
     <row r="94" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="B94" s="5">
         <v>46162.79269070602</v>
@@ -7126,13 +7138,13 @@
         <v>26</v>
       </c>
       <c r="N94" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="O94" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="O94" s="6" t="s">
-        <v>288</v>
-      </c>
       <c r="P94" s="6" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="Q94" s="6"/>
       <c r="R94" s="6"/>
@@ -7142,7 +7154,7 @@
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="8" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B95" s="9">
         <v>46162.79269707176</v>
@@ -7179,13 +7191,13 @@
         <v>26</v>
       </c>
       <c r="N95" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="O95" s="10" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="P95" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="Q95" s="10"/>
       <c r="R95" s="10"/>
@@ -7195,7 +7207,7 @@
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B96" s="5">
         <v>46162.792703576386</v>
@@ -7232,13 +7244,13 @@
         <v>26</v>
       </c>
       <c r="N96" s="6" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="O96" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="P96" s="6" t="s">
         <v>290</v>
-      </c>
-      <c r="P96" s="6" t="s">
-        <v>292</v>
       </c>
       <c r="Q96" s="6"/>
       <c r="R96" s="6"/>
@@ -7248,7 +7260,7 @@
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="8" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B97" s="9">
         <v>46162.79271046296</v>
@@ -7285,13 +7297,13 @@
         <v>26</v>
       </c>
       <c r="N97" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="O97" s="10" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="P97" s="10" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="Q97" s="10"/>
       <c r="R97" s="10"/>
@@ -7301,7 +7313,7 @@
     </row>
     <row r="98" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="4" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="B98" s="5">
         <v>46162.792744861115</v>
@@ -7311,7 +7323,7 @@
         <v>46164.691619942125</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>26</v>
@@ -7338,13 +7350,13 @@
         <v>26</v>
       </c>
       <c r="N98" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P98" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="Q98" s="5">
         <v>46317</v>
@@ -7364,7 +7376,7 @@
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="B99" s="9">
         <v>46162.79274982639</v>
@@ -7401,13 +7413,13 @@
         <v>26</v>
       </c>
       <c r="N99" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="O99" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="O99" s="10" t="s">
-        <v>299</v>
-      </c>
       <c r="P99" s="10" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="Q99" s="10"/>
       <c r="R99" s="10"/>
@@ -7417,7 +7429,7 @@
     </row>
     <row r="100" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B100" s="5">
         <v>46162.79275559028</v>
@@ -7454,13 +7466,13 @@
         <v>26</v>
       </c>
       <c r="N100" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="O100" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="O100" s="6" t="s">
-        <v>299</v>
-      </c>
       <c r="P100" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="Q100" s="6"/>
       <c r="R100" s="6"/>
@@ -7470,7 +7482,7 @@
     </row>
     <row r="101" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="8" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B101" s="9">
         <v>46162.79276118056</v>
@@ -7507,13 +7519,13 @@
         <v>26</v>
       </c>
       <c r="N101" s="10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="O101" s="10" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="P101" s="10" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="Q101" s="10"/>
       <c r="R101" s="10"/>
@@ -7523,7 +7535,7 @@
     </row>
     <row r="102" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B102" s="5">
         <v>46162.792767754625</v>
@@ -7560,13 +7572,13 @@
         <v>26</v>
       </c>
       <c r="N102" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="O102" s="6" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="P102" s="6" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="Q102" s="6"/>
       <c r="R102" s="6"/>
@@ -7576,7 +7588,7 @@
     </row>
     <row r="103" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="8" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B103" s="9">
         <v>46162.79285696759</v>
@@ -7586,7 +7598,7 @@
         <v>46164.69173954861</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
@@ -7613,13 +7625,13 @@
         <v>26</v>
       </c>
       <c r="N103" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O103" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P103" s="10" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="Q103" s="9">
         <v>46321</v>
@@ -7639,7 +7651,7 @@
     </row>
     <row r="104" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="B104" s="5">
         <v>46162.792862511575</v>
@@ -7676,13 +7688,13 @@
         <v>26</v>
       </c>
       <c r="N104" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="O104" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P104" s="6" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="Q104" s="6"/>
       <c r="R104" s="6"/>
@@ -7692,7 +7704,7 @@
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="8" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B105" s="9">
         <v>46162.792868125005</v>
@@ -7729,13 +7741,13 @@
         <v>26</v>
       </c>
       <c r="N105" s="10" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="O105" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P105" s="10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="Q105" s="10"/>
       <c r="R105" s="10"/>
@@ -7745,7 +7757,7 @@
     </row>
     <row r="106" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="B106" s="5">
         <v>46162.792873750004</v>
@@ -7782,13 +7794,13 @@
         <v>26</v>
       </c>
       <c r="N106" s="6" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="O106" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P106" s="6" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="Q106" s="6"/>
       <c r="R106" s="6"/>
@@ -7798,7 +7810,7 @@
     </row>
     <row r="107" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="8" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B107" s="9">
         <v>46162.7928793287</v>
@@ -7835,13 +7847,13 @@
         <v>26</v>
       </c>
       <c r="N107" s="10" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="O107" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P107" s="10" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="Q107" s="10"/>
       <c r="R107" s="10"/>
@@ -7851,7 +7863,7 @@
     </row>
     <row r="108" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="B108" s="5">
         <v>46162.792907696756</v>
@@ -7861,7 +7873,7 @@
         <v>46164.69185736111</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
@@ -7886,13 +7898,13 @@
         <v>26</v>
       </c>
       <c r="N108" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P108" s="6" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="Q108" s="5">
         <v>46323</v>
@@ -7912,7 +7924,7 @@
     </row>
     <row r="109" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="8" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="B109" s="9">
         <v>46162.79291289352</v>
@@ -7949,13 +7961,13 @@
         <v>26</v>
       </c>
       <c r="N109" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="O109" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P109" s="10" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="Q109" s="10"/>
       <c r="R109" s="10"/>
@@ -7965,7 +7977,7 @@
     </row>
     <row r="110" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="B110" s="5">
         <v>46162.79291758101</v>
@@ -8002,13 +8014,13 @@
         <v>26</v>
       </c>
       <c r="N110" s="6" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="O110" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P110" s="6" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="Q110" s="6"/>
       <c r="R110" s="6"/>
@@ -8018,7 +8030,7 @@
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="8" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B111" s="9">
         <v>46162.79292245371</v>
@@ -8055,13 +8067,13 @@
         <v>26</v>
       </c>
       <c r="N111" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="O111" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P111" s="10" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="Q111" s="10"/>
       <c r="R111" s="10"/>
@@ -8071,7 +8083,7 @@
     </row>
     <row r="112" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B112" s="5">
         <v>46162.79293256944</v>
@@ -8108,13 +8120,13 @@
         <v>26</v>
       </c>
       <c r="N112" s="6" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="O112" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P112" s="6" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="Q112" s="6"/>
       <c r="R112" s="6"/>
@@ -8124,7 +8136,7 @@
     </row>
     <row r="113" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="8" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B113" s="9">
         <v>46162.7930040625</v>
@@ -8134,7 +8146,7 @@
         <v>46164.68546163195</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>25</v>
@@ -8158,7 +8170,7 @@
         <v>26</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="P113" s="10" t="s">
         <v>26</v>
@@ -8171,7 +8183,7 @@
     </row>
     <row r="114" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="B114" s="5">
         <v>46162.79300806713</v>
@@ -8181,16 +8193,16 @@
         <v>46164.6922515162</v>
       </c>
       <c r="E114" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="F114" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G114" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="H114" s="6" t="s">
         <v>326</v>
-      </c>
-      <c r="F114" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G114" s="6" t="s">
-        <v>327</v>
-      </c>
-      <c r="H114" s="6" t="s">
-        <v>328</v>
       </c>
       <c r="I114" s="5">
         <v>46324</v>
@@ -8208,13 +8220,13 @@
         <v>26</v>
       </c>
       <c r="N114" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="P114" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="Q114" s="5">
         <v>46324</v>
@@ -8234,7 +8246,7 @@
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="8" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="B115" s="9">
         <v>46162.79301847222</v>
@@ -8250,10 +8262,10 @@
         <v>26</v>
       </c>
       <c r="G115" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H115" s="10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I115" s="9">
         <v>46324</v>
@@ -8271,13 +8283,13 @@
         <v>26</v>
       </c>
       <c r="N115" s="10" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="O115" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P115" s="10" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="Q115" s="10"/>
       <c r="R115" s="10"/>
@@ -8287,7 +8299,7 @@
     </row>
     <row r="116" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B116" s="5">
         <v>46162.79302525463</v>
@@ -8303,10 +8315,10 @@
         <v>26</v>
       </c>
       <c r="G116" s="6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H116" s="6" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I116" s="5">
         <v>46324</v>
@@ -8324,13 +8336,13 @@
         <v>26</v>
       </c>
       <c r="N116" s="6" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="O116" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P116" s="6" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="Q116" s="6"/>
       <c r="R116" s="6"/>
@@ -8340,7 +8352,7 @@
     </row>
     <row r="117" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="B117" s="9">
         <v>46162.79303010416</v>
@@ -8356,10 +8368,10 @@
         <v>26</v>
       </c>
       <c r="G117" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H117" s="10" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I117" s="9">
         <v>46324</v>
@@ -8377,13 +8389,13 @@
         <v>26</v>
       </c>
       <c r="N117" s="10" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="O117" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P117" s="10" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="Q117" s="10"/>
       <c r="R117" s="10"/>
@@ -8393,7 +8405,7 @@
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="B118" s="5">
         <v>46162.79303482639</v>
@@ -8409,10 +8421,10 @@
         <v>26</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="H118" s="6" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="I118" s="5">
         <v>46324</v>
@@ -8430,13 +8442,13 @@
         <v>26</v>
       </c>
       <c r="N118" s="6" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="O118" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="Q118" s="6"/>
       <c r="R118" s="6"/>
@@ -8446,7 +8458,7 @@
     </row>
     <row r="119" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="8" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="B119" s="9">
         <v>46162.79306296296</v>
@@ -8456,7 +8468,7 @@
         <v>46164.692368958335</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>26</v>
@@ -8483,13 +8495,13 @@
         <v>26</v>
       </c>
       <c r="N119" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="O119" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P119" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="Q119" s="9">
         <v>46325</v>
@@ -8509,7 +8521,7 @@
     </row>
     <row r="120" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B120" s="5">
         <v>46162.7930678125</v>
@@ -8546,13 +8558,13 @@
         <v>26</v>
       </c>
       <c r="N120" s="6" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="O120" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8562,7 +8574,7 @@
     </row>
     <row r="121" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="B121" s="9">
         <v>46162.793072280096</v>
@@ -8599,13 +8611,13 @@
         <v>26</v>
       </c>
       <c r="N121" s="10" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="O121" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P121" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="Q121" s="10"/>
       <c r="R121" s="10"/>
@@ -8615,7 +8627,7 @@
     </row>
     <row r="122" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="B122" s="5">
         <v>46162.79307696759</v>
@@ -8652,13 +8664,13 @@
         <v>26</v>
       </c>
       <c r="N122" s="6" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="O122" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8668,7 +8680,7 @@
     </row>
     <row r="123" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="8" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="B123" s="9">
         <v>46162.79308175926</v>
@@ -8705,13 +8717,13 @@
         <v>26</v>
       </c>
       <c r="N123" s="10" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="O123" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P123" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="Q123" s="10"/>
       <c r="R123" s="10"/>
@@ -8721,7 +8733,7 @@
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="B124" s="5">
         <v>46162.79314625</v>
@@ -8731,16 +8743,16 @@
         <v>46164.69248696759</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H124" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I124" s="5">
         <v>46328</v>
@@ -8758,13 +8770,13 @@
         <v>26</v>
       </c>
       <c r="N124" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P124" s="6" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="Q124" s="5">
         <v>46328</v>
@@ -8784,7 +8796,7 @@
     </row>
     <row r="125" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="8" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="B125" s="9">
         <v>46162.793151550926</v>
@@ -8800,10 +8812,10 @@
         <v>26</v>
       </c>
       <c r="G125" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H125" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I125" s="9">
         <v>46328</v>
@@ -8821,13 +8833,13 @@
         <v>26</v>
       </c>
       <c r="N125" s="10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="O125" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P125" s="10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="Q125" s="10"/>
       <c r="R125" s="10"/>
@@ -8837,7 +8849,7 @@
     </row>
     <row r="126" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="B126" s="5">
         <v>46162.79315885417</v>
@@ -8853,10 +8865,10 @@
         <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I126" s="5">
         <v>46328</v>
@@ -8874,13 +8886,13 @@
         <v>26</v>
       </c>
       <c r="N126" s="6" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="O126" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P126" s="6" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="Q126" s="6"/>
       <c r="R126" s="6"/>
@@ -8890,7 +8902,7 @@
     </row>
     <row r="127" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="8" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B127" s="9">
         <v>46162.79316501158</v>
@@ -8906,10 +8918,10 @@
         <v>26</v>
       </c>
       <c r="G127" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H127" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I127" s="9">
         <v>46328</v>
@@ -8927,13 +8939,13 @@
         <v>26</v>
       </c>
       <c r="N127" s="10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="O127" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P127" s="10" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="Q127" s="10"/>
       <c r="R127" s="10"/>
@@ -8943,7 +8955,7 @@
     </row>
     <row r="128" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="B128" s="5">
         <v>46162.79316986111</v>
@@ -8959,10 +8971,10 @@
         <v>26</v>
       </c>
       <c r="G128" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H128" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I128" s="5">
         <v>46328</v>
@@ -8980,13 +8992,13 @@
         <v>26</v>
       </c>
       <c r="N128" s="6" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="O128" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P128" s="6" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="Q128" s="6"/>
       <c r="R128" s="6"/>
@@ -8996,7 +9008,7 @@
     </row>
     <row r="129" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A129" s="8" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B129" s="9">
         <v>46162.79319725695</v>
@@ -9006,16 +9018,16 @@
         <v>46164.69262644676</v>
       </c>
       <c r="E129" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F129" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G129" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H129" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I129" s="9">
         <v>46329</v>
@@ -9033,13 +9045,13 @@
         <v>26</v>
       </c>
       <c r="N129" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="O129" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="P129" s="10" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="Q129" s="9">
         <v>46329</v>
@@ -9059,7 +9071,7 @@
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="B130" s="5">
         <v>46162.79320210648</v>
@@ -9075,10 +9087,10 @@
         <v>26</v>
       </c>
       <c r="G130" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H130" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I130" s="5">
         <v>46329</v>
@@ -9096,13 +9108,13 @@
         <v>26</v>
       </c>
       <c r="N130" s="6" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="O130" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P130" s="6" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="Q130" s="6"/>
       <c r="R130" s="6"/>
@@ -9112,7 +9124,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="B131" s="9">
         <v>46162.793206111106</v>
@@ -9128,10 +9140,10 @@
         <v>26</v>
       </c>
       <c r="G131" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H131" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I131" s="9">
         <v>46329</v>
@@ -9149,13 +9161,13 @@
         <v>26</v>
       </c>
       <c r="N131" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="O131" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P131" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="Q131" s="10"/>
       <c r="R131" s="10"/>
@@ -9165,7 +9177,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B132" s="5">
         <v>46162.7932099537</v>
@@ -9181,10 +9193,10 @@
         <v>26</v>
       </c>
       <c r="G132" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H132" s="6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I132" s="5">
         <v>46329</v>
@@ -9202,13 +9214,13 @@
         <v>26</v>
       </c>
       <c r="N132" s="6" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="O132" s="6" t="s">
         <v>189</v>
       </c>
       <c r="P132" s="6" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="Q132" s="6"/>
       <c r="R132" s="6"/>
@@ -9218,7 +9230,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="8" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="B133" s="9">
         <v>46162.79321400463</v>
@@ -9234,10 +9246,10 @@
         <v>26</v>
       </c>
       <c r="G133" s="10" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H133" s="10" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="I133" s="9">
         <v>46329</v>
@@ -9255,13 +9267,13 @@
         <v>26</v>
       </c>
       <c r="N133" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="O133" s="10" t="s">
         <v>189</v>
       </c>
       <c r="P133" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="Q133" s="10"/>
       <c r="R133" s="10"/>
@@ -9271,7 +9283,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="B134" s="5">
         <v>46162.79323766204</v>
@@ -9281,7 +9293,7 @@
         <v>46164.685922812496</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>25</v>
@@ -9305,7 +9317,7 @@
         <v>26</v>
       </c>
       <c r="O134" s="6" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="P134" s="6" t="s">
         <v>26</v>
@@ -9318,7 +9330,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="8" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B135" s="9">
         <v>46162.79324063657</v>
@@ -9328,16 +9340,16 @@
         <v>46164.69269384259</v>
       </c>
       <c r="E135" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="F135" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G135" s="10" t="s">
+        <v>363</v>
+      </c>
+      <c r="H135" s="10" t="s">
         <v>364</v>
-      </c>
-      <c r="F135" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G135" s="10" t="s">
-        <v>365</v>
-      </c>
-      <c r="H135" s="10" t="s">
-        <v>366</v>
       </c>
       <c r="I135" s="9">
         <v>46330</v>
@@ -9355,13 +9367,13 @@
         <v>26</v>
       </c>
       <c r="N135" s="10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O135" s="10" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="P135" s="10" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="Q135" s="9">
         <v>46330</v>
@@ -9381,7 +9393,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="B136" s="5">
         <v>46162.79324528935</v>
@@ -9391,7 +9403,7 @@
         <v>46197.77680827546</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="F136" s="6" t="s">
         <v>26</v>
@@ -9418,13 +9430,13 @@
         <v>26</v>
       </c>
       <c r="N136" s="6" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="O136" s="6" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="P136" s="6" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="Q136" s="5">
         <v>46330</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-09-12 13:17 Chile
</commit_message>
<xml_diff>
--- a/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
+++ b/data/50001553 - ZITRON COLOMBIA ARIS OT4326.xlsx
@@ -364,163 +364,163 @@
     <t>Fabricación Alabe,Generación OC Alabe</t>
   </si>
   <si>
+    <t>1214982580348412</t>
+  </si>
+  <si>
+    <t>Generación OC Alabe</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe,Alabe</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
+  </si>
+  <si>
+    <t>1214982387972692</t>
+  </si>
+  <si>
+    <t>Fabricación Alabe</t>
+  </si>
+  <si>
+    <t>Alabe,Recepcion Alabe</t>
+  </si>
+  <si>
+    <t>1214982387972712</t>
+  </si>
+  <si>
+    <t>rodete</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete,Fabricación Rodete</t>
+  </si>
+  <si>
+    <t>1214982387972761</t>
+  </si>
+  <si>
+    <t>Generación OC Rodete</t>
+  </si>
+  <si>
+    <t>rodete,Fabricación Rodete</t>
+  </si>
+  <si>
+    <t>1214982387972781</t>
+  </si>
+  <si>
+    <t>Fabricación Rodete</t>
+  </si>
+  <si>
+    <t>rodete,Recepcion Rodete</t>
+  </si>
+  <si>
+    <t>1214982387980169</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>Generación OC motor,Fabricación motor,Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>1214982508487948</t>
+  </si>
+  <si>
+    <t>Generación OC motor</t>
+  </si>
+  <si>
+    <t>Motor,Fabricación motor,Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>1214982508487968</t>
+  </si>
+  <si>
+    <t>Fabricación motor</t>
+  </si>
+  <si>
+    <t>Recepcion motor,Motor</t>
+  </si>
+  <si>
+    <t>1214982595218704</t>
+  </si>
+  <si>
+    <t>Planos motor proveedor</t>
+  </si>
+  <si>
+    <t>Motor,Planos definitivos</t>
+  </si>
+  <si>
+    <t>1214982595218724</t>
+  </si>
+  <si>
+    <t>Materiales corte Laser</t>
+  </si>
+  <si>
+    <t>Yerlia Ayleen Castillo Diaz</t>
+  </si>
+  <si>
+    <t>yerlia.castillo@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC materiales corte Laser,Fabricacion Corte Laser </t>
+  </si>
+  <si>
+    <t>1214982558049172</t>
+  </si>
+  <si>
+    <t>Generación OC materiales corte Laser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiales corte Laser,Fabricacion Corte Laser </t>
+  </si>
+  <si>
+    <t>1214982595219177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricacion Corte Laser </t>
+  </si>
+  <si>
+    <t>Recepcion materiales corte laser,Materiales corte Laser</t>
+  </si>
+  <si>
+    <t>1214982595219197</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiales Corte Plasma </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Corte Plasma ,Fabricación Corte Plasma </t>
+  </si>
+  <si>
+    <t>1214982558071444</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Materiales Corte Plasma ,Fabricación Corte Plasma </t>
+  </si>
+  <si>
+    <t>1214982558071461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Corte Plasma </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recepcion Materiales corte plasma,Materiales Corte Plasma </t>
+  </si>
+  <si>
+    <t>1214995680413404</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación Externa </t>
+  </si>
+  <si>
+    <t>Rosemary Singh</t>
+  </si>
+  <si>
+    <t>rosemary.singh@zitron.com</t>
+  </si>
+  <si>
+    <t>Fabricación estructura proveedor externo,Generacion OC Fabricación Externa</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1214982580348412</t>
-  </si>
-  <si>
-    <t>Generación OC Alabe</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe,Alabe</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
-  </si>
-  <si>
-    <t>1214982387972692</t>
-  </si>
-  <si>
-    <t>Fabricación Alabe</t>
-  </si>
-  <si>
-    <t>Alabe,Recepcion Alabe</t>
-  </si>
-  <si>
-    <t>1214982387972712</t>
-  </si>
-  <si>
-    <t>rodete</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete,Fabricación Rodete</t>
-  </si>
-  <si>
-    <t>1214982387972761</t>
-  </si>
-  <si>
-    <t>Generación OC Rodete</t>
-  </si>
-  <si>
-    <t>rodete,Fabricación Rodete</t>
-  </si>
-  <si>
-    <t>1214982387972781</t>
-  </si>
-  <si>
-    <t>Fabricación Rodete</t>
-  </si>
-  <si>
-    <t>rodete,Recepcion Rodete</t>
-  </si>
-  <si>
-    <t>1214982387980169</t>
-  </si>
-  <si>
-    <t>Motor</t>
-  </si>
-  <si>
-    <t>Generación OC motor,Fabricación motor,Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>1214982508487948</t>
-  </si>
-  <si>
-    <t>Generación OC motor</t>
-  </si>
-  <si>
-    <t>Motor,Fabricación motor,Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>1214982508487968</t>
-  </si>
-  <si>
-    <t>Fabricación motor</t>
-  </si>
-  <si>
-    <t>Recepcion motor,Motor</t>
-  </si>
-  <si>
-    <t>1214982595218704</t>
-  </si>
-  <si>
-    <t>Planos motor proveedor</t>
-  </si>
-  <si>
-    <t>Motor,Planos definitivos</t>
-  </si>
-  <si>
-    <t>1214982595218724</t>
-  </si>
-  <si>
-    <t>Materiales corte Laser</t>
-  </si>
-  <si>
-    <t>Yerlia Ayleen Castillo Diaz</t>
-  </si>
-  <si>
-    <t>yerlia.castillo@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC materiales corte Laser,Fabricacion Corte Laser </t>
-  </si>
-  <si>
-    <t>1214982558049172</t>
-  </si>
-  <si>
-    <t>Generación OC materiales corte Laser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Materiales corte Laser,Fabricacion Corte Laser </t>
-  </si>
-  <si>
-    <t>1214982595219177</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricacion Corte Laser </t>
-  </si>
-  <si>
-    <t>Recepcion materiales corte laser,Materiales corte Laser</t>
-  </si>
-  <si>
-    <t>1214982595219197</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Materiales Corte Plasma </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Corte Plasma ,Fabricación Corte Plasma </t>
-  </si>
-  <si>
-    <t>1214982558071444</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Materiales Corte Plasma ,Fabricación Corte Plasma </t>
-  </si>
-  <si>
-    <t>1214982558071461</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Corte Plasma </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recepcion Materiales corte plasma,Materiales Corte Plasma </t>
-  </si>
-  <si>
-    <t>1214995680413404</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación Externa </t>
-  </si>
-  <si>
-    <t>Rosemary Singh</t>
-  </si>
-  <si>
-    <t>rosemary.singh@zitron.com</t>
-  </si>
-  <si>
-    <t>Fabricación estructura proveedor externo,Generacion OC Fabricación Externa</t>
   </si>
   <si>
     <t>1214995680413416</t>
@@ -2926,7 +2926,7 @@
         <v>46198.68595238426</v>
       </c>
       <c r="D22" s="5">
-        <v>46269.176564849535</v>
+        <v>46277.14165576389</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>93</v>
@@ -2970,8 +2970,8 @@
       <c r="R22" s="5">
         <v>46276</v>
       </c>
-      <c r="S22" s="12" t="s">
-        <v>97</v>
+      <c r="S22" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="T22" s="6">
         <v>1</v>
@@ -2982,7 +2982,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B23" s="9">
         <v>46162.791964375</v>
@@ -2994,7 +2994,7 @@
         <v>46198.68590748843</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
@@ -3027,7 +3027,7 @@
         <v>68</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q23" s="10"/>
       <c r="R23" s="10"/>
@@ -3038,12 +3038,12 @@
         <v>0</v>
       </c>
       <c r="U23" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24" s="5">
         <v>46162.79196883102</v>
@@ -3055,7 +3055,7 @@
         <v>46198.6859406713</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
@@ -3085,10 +3085,10 @@
         <v>93</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
@@ -3099,12 +3099,12 @@
         <v>0</v>
       </c>
       <c r="U24" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B25" s="9">
         <v>46162.79197329861</v>
@@ -3116,7 +3116,7 @@
         <v>46212.65520907407</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
@@ -3146,7 +3146,7 @@
         <v>90</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P25" s="10" t="s">
         <v>90</v>
@@ -3169,7 +3169,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B26" s="5">
         <v>46162.791977500005</v>
@@ -3181,7 +3181,7 @@
         <v>46212.65503678241</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
@@ -3208,13 +3208,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O26" s="6" t="s">
         <v>71</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
@@ -3225,12 +3225,12 @@
         <v>0</v>
       </c>
       <c r="U26" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B27" s="9">
         <v>46162.79198199074</v>
@@ -3242,7 +3242,7 @@
         <v>46212.65507065972</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
@@ -3269,13 +3269,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
@@ -3286,12 +3286,12 @@
         <v>0</v>
       </c>
       <c r="U27" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B28" s="5">
         <v>46162.79198653935</v>
@@ -3303,7 +3303,7 @@
         <v>46198.68573546296</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
@@ -3333,7 +3333,7 @@
         <v>90</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>90</v>
@@ -3356,7 +3356,7 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B29" s="9">
         <v>46162.79199082176</v>
@@ -3368,7 +3368,7 @@
         <v>46198.68152484954</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
@@ -3395,13 +3395,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O29" s="10" t="s">
         <v>65</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="Q29" s="10"/>
       <c r="R29" s="10"/>
@@ -3412,12 +3412,12 @@
         <v>0</v>
       </c>
       <c r="U29" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B30" s="5">
         <v>46162.791995312495</v>
@@ -3429,7 +3429,7 @@
         <v>46198.68567791667</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
@@ -3456,13 +3456,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
@@ -3473,12 +3473,12 @@
         <v>0</v>
       </c>
       <c r="U30" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B31" s="9">
         <v>46162.79199990741</v>
@@ -3490,7 +3490,7 @@
         <v>46198.68156315973</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
@@ -3517,13 +3517,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
@@ -3534,12 +3534,12 @@
         <v>0</v>
       </c>
       <c r="U31" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B32" s="5">
         <v>46162.792004421295</v>
@@ -3551,16 +3551,16 @@
         <v>46252.179607199076</v>
       </c>
       <c r="E32" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G32" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F32" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G32" s="6" t="s">
+      <c r="H32" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="I32" s="5">
         <v>46239</v>
@@ -3581,7 +3581,7 @@
         <v>90</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P32" s="6" t="s">
         <v>90</v>
@@ -3604,7 +3604,7 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B33" s="9">
         <v>46162.79200878472</v>
@@ -3616,16 +3616,16 @@
         <v>46205.6112640625</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="H33" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="I33" s="9">
         <v>46239</v>
@@ -3643,13 +3643,13 @@
         <v>26</v>
       </c>
       <c r="N33" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O33" s="10" t="s">
         <v>77</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Q33" s="10"/>
       <c r="R33" s="10"/>
@@ -3660,12 +3660,12 @@
         <v>0</v>
       </c>
       <c r="U33" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B34" s="5">
         <v>46162.792013391205</v>
@@ -3677,16 +3677,16 @@
         <v>46209.81741092593</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="I34" s="5">
         <v>46241</v>
@@ -3704,13 +3704,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -3721,12 +3721,12 @@
         <v>0</v>
       </c>
       <c r="U34" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B35" s="9">
         <v>46162.79201809027</v>
@@ -3738,16 +3738,16 @@
         <v>46252.17960721065</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="I35" s="9">
         <v>46239</v>
@@ -3768,7 +3768,7 @@
         <v>90</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P35" s="10" t="s">
         <v>26</v>
@@ -3791,7 +3791,7 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B36" s="5">
         <v>46162.79207501157</v>
@@ -3809,10 +3809,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="I36" s="5">
         <v>46239</v>
@@ -3830,13 +3830,13 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>81</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
@@ -3846,7 +3846,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B37" s="9">
         <v>46162.79208025463</v>
@@ -3858,16 +3858,16 @@
         <v>46209.817526388884</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="I37" s="9">
         <v>46241</v>
@@ -3885,13 +3885,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O37" s="10" t="s">
         <v>82</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3901,7 +3901,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B38" s="5">
         <v>46162.792085</v>
@@ -3913,16 +3913,16 @@
         <v>46272.13554642361</v>
       </c>
       <c r="E38" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G38" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="F38" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G38" s="6" t="s">
+      <c r="H38" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="I38" s="5">
         <v>46239</v>
@@ -3943,7 +3943,7 @@
         <v>90</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="P38" s="6" t="s">
         <v>26</v>
@@ -3955,7 +3955,7 @@
         <v>46279</v>
       </c>
       <c r="S38" s="12" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="T38" s="6">
         <v>1</v>
@@ -3984,10 +3984,10 @@
         <v>26</v>
       </c>
       <c r="G39" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="H39" s="10" t="s">
         <v>147</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>148</v>
       </c>
       <c r="I39" s="9">
         <v>46239</v>
@@ -4005,7 +4005,7 @@
         <v>26</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O39" s="10" t="s">
         <v>87</v>
@@ -4039,10 +4039,10 @@
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="I40" s="5">
         <v>46248</v>
@@ -4060,7 +4060,7 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>88</v>
@@ -4113,7 +4113,7 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O41" s="10" t="s">
         <v>153</v>
@@ -4147,10 +4147,10 @@
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H42" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="I42" s="5">
         <v>46239</v>
@@ -4212,10 +4212,10 @@
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>128</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>129</v>
       </c>
       <c r="I43" s="9">
         <v>46239</v>
@@ -4267,10 +4267,10 @@
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="I44" s="5">
         <v>46241</v>
@@ -4924,7 +4924,7 @@
         <v>195</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="P55" s="10" t="s">
         <v>201</v>
@@ -5054,7 +5054,7 @@
         <v>195</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="P57" s="10" t="s">
         <v>207</v>
@@ -6271,7 +6271,7 @@
         <v>195</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>252</v>
@@ -6336,7 +6336,7 @@
         <v>195</v>
       </c>
       <c r="O79" s="10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P79" s="10" t="s">
         <v>255</v>
@@ -6348,7 +6348,7 @@
         <v>46280</v>
       </c>
       <c r="S79" s="12" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="T79" s="10">
         <v>1</v>
@@ -6401,7 +6401,7 @@
         <v>195</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>204</v>
@@ -6476,7 +6476,7 @@
         <v>46281</v>
       </c>
       <c r="S81" s="12" t="s">
-        <v>97</v>
+        <v>149</v>
       </c>
       <c r="T81" s="10">
         <v>0</v>
@@ -8305,7 +8305,7 @@
         <v>0</v>
       </c>
       <c r="U114" s="11" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="115" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>